<commit_message>
feat: agregar funcionalidad para incluir una hoja de anexo en la generación de la nómina de pago, mejorando la presentación de datos administrativos y asegurando la carga de plantilla correspondiente
</commit_message>
<xml_diff>
--- a/src/core/excel/templates/ANEXO NOMINA DE PAGO PERSONAL ADMINISTRATIVO.xlsx
+++ b/src/core/excel/templates/ANEXO NOMINA DE PAGO PERSONAL ADMINISTRATIVO.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\david\OneDrive\Documentos\Codigo\san-miguel-porres-backend\src\core\excel\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A622B1E4-593D-483B-9481-A07C1D4FD284}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0E9D5D8-1D71-4DD6-BD27-F56BF7AEBB8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -532,15 +532,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
@@ -550,15 +541,6 @@
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
@@ -576,15 +558,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -600,122 +573,17 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -738,12 +606,6 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="4" fontId="12" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -765,19 +627,157 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="17" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="16" fillId="0" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="17" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="4" fontId="16" fillId="0" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -2183,31 +2183,31 @@
       <c r="L2" s="8"/>
       <c r="M2" s="8"/>
       <c r="N2" s="8"/>
-      <c r="O2" s="10" t="s">
+      <c r="O2" s="88" t="s">
         <v>4</v>
       </c>
-      <c r="P2" s="11"/>
-      <c r="Q2" s="11"/>
-      <c r="R2" s="11"/>
-      <c r="S2" s="11"/>
-      <c r="T2" s="11"/>
-      <c r="U2" s="11"/>
-      <c r="V2" s="11"/>
-      <c r="W2" s="11"/>
-      <c r="X2" s="11"/>
-      <c r="Y2" s="12"/>
+      <c r="P2" s="89"/>
+      <c r="Q2" s="89"/>
+      <c r="R2" s="89"/>
+      <c r="S2" s="89"/>
+      <c r="T2" s="89"/>
+      <c r="U2" s="89"/>
+      <c r="V2" s="89"/>
+      <c r="W2" s="89"/>
+      <c r="X2" s="89"/>
+      <c r="Y2" s="90"/>
       <c r="Z2" s="1"/>
       <c r="AA2" s="1"/>
       <c r="AB2" s="1"/>
     </row>
     <row r="3" spans="1:28" ht="23.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="14"/>
-      <c r="C3" s="14"/>
-      <c r="D3" s="14"/>
-      <c r="E3" s="15"/>
+      <c r="B3" s="11"/>
+      <c r="C3" s="11"/>
+      <c r="D3" s="11"/>
+      <c r="E3" s="12"/>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
       <c r="H3" s="1"/>
@@ -2217,59 +2217,59 @@
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
       <c r="N3" s="1"/>
-      <c r="O3" s="16" t="s">
+      <c r="O3" s="91" t="s">
         <v>6</v>
       </c>
-      <c r="P3" s="17"/>
-      <c r="Q3" s="17"/>
-      <c r="R3" s="17"/>
-      <c r="S3" s="17"/>
-      <c r="T3" s="17"/>
-      <c r="U3" s="17"/>
-      <c r="V3" s="17"/>
-      <c r="W3" s="17"/>
-      <c r="X3" s="17"/>
-      <c r="Y3" s="18"/>
+      <c r="P3" s="92"/>
+      <c r="Q3" s="92"/>
+      <c r="R3" s="92"/>
+      <c r="S3" s="92"/>
+      <c r="T3" s="92"/>
+      <c r="U3" s="92"/>
+      <c r="V3" s="92"/>
+      <c r="W3" s="92"/>
+      <c r="X3" s="92"/>
+      <c r="Y3" s="93"/>
       <c r="Z3" s="1"/>
       <c r="AA3" s="1"/>
       <c r="AB3" s="1"/>
     </row>
     <row r="4" spans="1:28" ht="23.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="20"/>
-      <c r="C4" s="20"/>
-      <c r="D4" s="21"/>
-      <c r="E4" s="22"/>
-      <c r="F4" s="23"/>
-      <c r="G4" s="23"/>
-      <c r="H4" s="23"/>
-      <c r="I4" s="23"/>
-      <c r="J4" s="23"/>
-      <c r="K4" s="24"/>
-      <c r="L4" s="24"/>
-      <c r="M4" s="24"/>
-      <c r="N4" s="24"/>
-      <c r="O4" s="25" t="s">
+      <c r="B4" s="14"/>
+      <c r="C4" s="14"/>
+      <c r="D4" s="15"/>
+      <c r="E4" s="16"/>
+      <c r="F4" s="17"/>
+      <c r="G4" s="17"/>
+      <c r="H4" s="17"/>
+      <c r="I4" s="17"/>
+      <c r="J4" s="17"/>
+      <c r="K4" s="18"/>
+      <c r="L4" s="18"/>
+      <c r="M4" s="18"/>
+      <c r="N4" s="18"/>
+      <c r="O4" s="94" t="s">
         <v>8</v>
       </c>
-      <c r="P4" s="26"/>
-      <c r="Q4" s="26"/>
-      <c r="R4" s="26"/>
-      <c r="S4" s="26"/>
-      <c r="T4" s="26"/>
-      <c r="U4" s="26"/>
-      <c r="V4" s="26"/>
-      <c r="W4" s="26"/>
-      <c r="X4" s="26"/>
-      <c r="Y4" s="27"/>
+      <c r="P4" s="95"/>
+      <c r="Q4" s="95"/>
+      <c r="R4" s="95"/>
+      <c r="S4" s="95"/>
+      <c r="T4" s="95"/>
+      <c r="U4" s="95"/>
+      <c r="V4" s="95"/>
+      <c r="W4" s="95"/>
+      <c r="X4" s="95"/>
+      <c r="Y4" s="96"/>
       <c r="Z4" s="1"/>
       <c r="AA4" s="1"/>
       <c r="AB4" s="1"/>
     </row>
     <row r="5" spans="1:28" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="28"/>
+      <c r="A5" s="19"/>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
@@ -2293,846 +2293,825 @@
       <c r="V5" s="1"/>
       <c r="W5" s="1"/>
       <c r="X5" s="1"/>
-      <c r="Y5" s="29"/>
+      <c r="Y5" s="20"/>
       <c r="Z5" s="1"/>
       <c r="AA5" s="1"/>
       <c r="AB5" s="1"/>
     </row>
     <row r="6" spans="1:28" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="30"/>
-      <c r="B6" s="31">
+      <c r="A6" s="21"/>
+      <c r="B6" s="22">
         <v>1</v>
       </c>
-      <c r="C6" s="32">
+      <c r="C6" s="23">
         <v>2</v>
       </c>
-      <c r="D6" s="32">
+      <c r="D6" s="23">
         <v>3</v>
       </c>
-      <c r="E6" s="32">
+      <c r="E6" s="23">
         <v>4</v>
       </c>
-      <c r="F6" s="33">
+      <c r="F6" s="77">
         <v>5</v>
       </c>
-      <c r="G6" s="34"/>
-      <c r="H6" s="33">
+      <c r="G6" s="79"/>
+      <c r="H6" s="77">
         <v>6</v>
       </c>
-      <c r="I6" s="34"/>
-      <c r="J6" s="32">
+      <c r="I6" s="79"/>
+      <c r="J6" s="23">
         <v>7</v>
       </c>
-      <c r="K6" s="33">
+      <c r="K6" s="77">
         <v>8</v>
       </c>
-      <c r="L6" s="35"/>
-      <c r="M6" s="35"/>
-      <c r="N6" s="35"/>
-      <c r="O6" s="34"/>
-      <c r="P6" s="32">
+      <c r="L6" s="78"/>
+      <c r="M6" s="78"/>
+      <c r="N6" s="78"/>
+      <c r="O6" s="79"/>
+      <c r="P6" s="23">
         <v>9</v>
       </c>
-      <c r="Q6" s="32" t="s">
+      <c r="Q6" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="R6" s="32" t="s">
+      <c r="R6" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="S6" s="32" t="s">
+      <c r="S6" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="T6" s="32" t="s">
+      <c r="T6" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="U6" s="32" t="s">
+      <c r="U6" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="V6" s="32" t="s">
+      <c r="V6" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="W6" s="32" t="s">
+      <c r="W6" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="X6" s="32" t="s">
+      <c r="X6" s="23" t="s">
         <v>16</v>
       </c>
-      <c r="Y6" s="32">
+      <c r="Y6" s="23">
         <v>4</v>
       </c>
-      <c r="Z6" s="36"/>
-      <c r="AA6" s="36"/>
-      <c r="AB6" s="36"/>
+      <c r="Z6" s="24"/>
+      <c r="AA6" s="24"/>
+      <c r="AB6" s="24"/>
     </row>
     <row r="7" spans="1:28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="37" t="s">
+      <c r="A7" s="73" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="38" t="s">
+      <c r="B7" s="80" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="39" t="s">
+      <c r="C7" s="82" t="s">
         <v>19</v>
       </c>
-      <c r="D7" s="39"/>
-      <c r="E7" s="40" t="s">
+      <c r="D7" s="82"/>
+      <c r="E7" s="84" t="s">
         <v>20</v>
       </c>
-      <c r="F7" s="41" t="s">
+      <c r="F7" s="61" t="s">
         <v>21</v>
       </c>
-      <c r="G7" s="42"/>
-      <c r="H7" s="41" t="s">
+      <c r="G7" s="86"/>
+      <c r="H7" s="61" t="s">
         <v>22</v>
       </c>
-      <c r="I7" s="43"/>
-      <c r="J7" s="44" t="s">
+      <c r="I7" s="62"/>
+      <c r="J7" s="65" t="s">
         <v>23</v>
       </c>
-      <c r="K7" s="45" t="s">
+      <c r="K7" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="L7" s="46"/>
-      <c r="M7" s="46"/>
-      <c r="N7" s="46"/>
-      <c r="O7" s="47"/>
-      <c r="P7" s="48"/>
-      <c r="Q7" s="49" t="s">
+      <c r="L7" s="68"/>
+      <c r="M7" s="68"/>
+      <c r="N7" s="68"/>
+      <c r="O7" s="69"/>
+      <c r="P7" s="25"/>
+      <c r="Q7" s="53" t="s">
         <v>25</v>
       </c>
-      <c r="R7" s="49" t="s">
+      <c r="R7" s="53" t="s">
         <v>26</v>
       </c>
-      <c r="S7" s="49" t="s">
+      <c r="S7" s="53" t="s">
         <v>27</v>
       </c>
-      <c r="T7" s="49" t="s">
+      <c r="T7" s="53" t="s">
         <v>28</v>
       </c>
-      <c r="U7" s="50" t="s">
+      <c r="U7" s="55" t="s">
         <v>29</v>
       </c>
-      <c r="V7" s="50" t="s">
+      <c r="V7" s="55" t="s">
         <v>30</v>
       </c>
-      <c r="W7" s="49" t="s">
+      <c r="W7" s="53" t="s">
         <v>31</v>
       </c>
-      <c r="X7" s="51" t="s">
+      <c r="X7" s="57" t="s">
         <v>32</v>
       </c>
-      <c r="Y7" s="52" t="s">
+      <c r="Y7" s="59" t="s">
         <v>33</v>
       </c>
-      <c r="Z7" s="53"/>
-      <c r="AA7" s="53"/>
-      <c r="AB7" s="53"/>
+      <c r="Z7" s="26"/>
+      <c r="AA7" s="26"/>
+      <c r="AB7" s="26"/>
     </row>
     <row r="8" spans="1:28" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="54"/>
-      <c r="B8" s="55"/>
-      <c r="C8" s="56"/>
-      <c r="D8" s="56"/>
-      <c r="E8" s="57"/>
-      <c r="F8" s="58"/>
-      <c r="G8" s="59"/>
-      <c r="H8" s="58"/>
-      <c r="I8" s="60"/>
-      <c r="J8" s="61"/>
-      <c r="K8" s="62"/>
-      <c r="L8" s="63"/>
-      <c r="M8" s="63"/>
-      <c r="N8" s="63"/>
-      <c r="O8" s="64"/>
-      <c r="P8" s="65"/>
-      <c r="Q8" s="66"/>
-      <c r="R8" s="66"/>
-      <c r="S8" s="66"/>
-      <c r="T8" s="66"/>
-      <c r="U8" s="67"/>
-      <c r="V8" s="67"/>
-      <c r="W8" s="66"/>
-      <c r="X8" s="68"/>
-      <c r="Y8" s="69"/>
-      <c r="Z8" s="53"/>
-      <c r="AA8" s="53"/>
-      <c r="AB8" s="53"/>
+      <c r="A8" s="74"/>
+      <c r="B8" s="81"/>
+      <c r="C8" s="83"/>
+      <c r="D8" s="83"/>
+      <c r="E8" s="85"/>
+      <c r="F8" s="63"/>
+      <c r="G8" s="87"/>
+      <c r="H8" s="63"/>
+      <c r="I8" s="64"/>
+      <c r="J8" s="66"/>
+      <c r="K8" s="70"/>
+      <c r="L8" s="71"/>
+      <c r="M8" s="71"/>
+      <c r="N8" s="71"/>
+      <c r="O8" s="72"/>
+      <c r="P8" s="27"/>
+      <c r="Q8" s="54"/>
+      <c r="R8" s="54"/>
+      <c r="S8" s="54"/>
+      <c r="T8" s="54"/>
+      <c r="U8" s="56"/>
+      <c r="V8" s="56"/>
+      <c r="W8" s="54"/>
+      <c r="X8" s="58"/>
+      <c r="Y8" s="60"/>
+      <c r="Z8" s="26"/>
+      <c r="AA8" s="26"/>
+      <c r="AB8" s="26"/>
     </row>
     <row r="9" spans="1:28" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="54"/>
-      <c r="B9" s="55"/>
-      <c r="C9" s="56"/>
-      <c r="D9" s="56"/>
-      <c r="E9" s="57"/>
-      <c r="F9" s="44" t="s">
+      <c r="A9" s="74"/>
+      <c r="B9" s="81"/>
+      <c r="C9" s="83"/>
+      <c r="D9" s="83"/>
+      <c r="E9" s="85"/>
+      <c r="F9" s="65" t="s">
         <v>34</v>
       </c>
-      <c r="G9" s="44" t="s">
+      <c r="G9" s="65" t="s">
         <v>35</v>
       </c>
-      <c r="H9" s="37" t="s">
+      <c r="H9" s="73" t="s">
         <v>36</v>
       </c>
-      <c r="I9" s="70" t="s">
+      <c r="I9" s="75" t="s">
         <v>37</v>
       </c>
-      <c r="J9" s="61"/>
-      <c r="K9" s="37" t="s">
+      <c r="J9" s="66"/>
+      <c r="K9" s="73" t="s">
         <v>38</v>
       </c>
-      <c r="L9" s="33" t="s">
+      <c r="L9" s="77" t="s">
         <v>39</v>
       </c>
-      <c r="M9" s="35"/>
-      <c r="N9" s="35"/>
-      <c r="O9" s="34"/>
-      <c r="P9" s="65"/>
-      <c r="Q9" s="66"/>
-      <c r="R9" s="66"/>
-      <c r="S9" s="66"/>
-      <c r="T9" s="66"/>
-      <c r="U9" s="67"/>
-      <c r="V9" s="67"/>
-      <c r="W9" s="66"/>
-      <c r="X9" s="68"/>
-      <c r="Y9" s="69"/>
-      <c r="Z9" s="53"/>
-      <c r="AA9" s="53"/>
-      <c r="AB9" s="53"/>
+      <c r="M9" s="78"/>
+      <c r="N9" s="78"/>
+      <c r="O9" s="79"/>
+      <c r="P9" s="27"/>
+      <c r="Q9" s="54"/>
+      <c r="R9" s="54"/>
+      <c r="S9" s="54"/>
+      <c r="T9" s="54"/>
+      <c r="U9" s="56"/>
+      <c r="V9" s="56"/>
+      <c r="W9" s="54"/>
+      <c r="X9" s="58"/>
+      <c r="Y9" s="60"/>
+      <c r="Z9" s="26"/>
+      <c r="AA9" s="26"/>
+      <c r="AB9" s="26"/>
     </row>
     <row r="10" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="54"/>
-      <c r="B10" s="55"/>
-      <c r="C10" s="56"/>
-      <c r="D10" s="56"/>
-      <c r="E10" s="57"/>
-      <c r="F10" s="61"/>
-      <c r="G10" s="61"/>
-      <c r="H10" s="54"/>
-      <c r="I10" s="71"/>
-      <c r="J10" s="61"/>
-      <c r="K10" s="54"/>
-      <c r="L10" s="72" t="s">
+      <c r="A10" s="74"/>
+      <c r="B10" s="81"/>
+      <c r="C10" s="83"/>
+      <c r="D10" s="83"/>
+      <c r="E10" s="85"/>
+      <c r="F10" s="66"/>
+      <c r="G10" s="66"/>
+      <c r="H10" s="74"/>
+      <c r="I10" s="76"/>
+      <c r="J10" s="66"/>
+      <c r="K10" s="74"/>
+      <c r="L10" s="28" t="s">
         <v>40</v>
       </c>
-      <c r="M10" s="72" t="s">
+      <c r="M10" s="28" t="s">
         <v>41</v>
       </c>
-      <c r="N10" s="72" t="s">
+      <c r="N10" s="28" t="s">
         <v>42</v>
       </c>
-      <c r="O10" s="72" t="s">
+      <c r="O10" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="P10" s="65"/>
-      <c r="Q10" s="66"/>
-      <c r="R10" s="66"/>
-      <c r="S10" s="66"/>
-      <c r="T10" s="66"/>
-      <c r="U10" s="67"/>
-      <c r="V10" s="67"/>
-      <c r="W10" s="66"/>
-      <c r="X10" s="68"/>
-      <c r="Y10" s="69"/>
-      <c r="Z10" s="53"/>
-      <c r="AA10" s="53"/>
-      <c r="AB10" s="53"/>
+      <c r="P10" s="27"/>
+      <c r="Q10" s="54"/>
+      <c r="R10" s="54"/>
+      <c r="S10" s="54"/>
+      <c r="T10" s="54"/>
+      <c r="U10" s="56"/>
+      <c r="V10" s="56"/>
+      <c r="W10" s="54"/>
+      <c r="X10" s="58"/>
+      <c r="Y10" s="60"/>
+      <c r="Z10" s="26"/>
+      <c r="AA10" s="26"/>
+      <c r="AB10" s="26"/>
     </row>
     <row r="11" spans="1:28" ht="48" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="73"/>
-      <c r="B11" s="73"/>
-      <c r="C11" s="73"/>
-      <c r="D11" s="73"/>
-      <c r="E11" s="73"/>
-      <c r="F11" s="73"/>
-      <c r="G11" s="73"/>
-      <c r="H11" s="74"/>
-      <c r="I11" s="73"/>
-      <c r="J11" s="74"/>
-      <c r="K11" s="75"/>
-      <c r="L11" s="76"/>
-      <c r="M11" s="73"/>
-      <c r="N11" s="73"/>
-      <c r="O11" s="73"/>
-      <c r="P11" s="73"/>
-      <c r="Q11" s="77"/>
-      <c r="R11" s="77"/>
-      <c r="S11" s="77"/>
-      <c r="T11" s="77"/>
-      <c r="U11" s="77"/>
-      <c r="V11" s="77"/>
-      <c r="W11" s="77"/>
-      <c r="X11" s="77"/>
-      <c r="Y11" s="77"/>
-      <c r="Z11" s="53"/>
-      <c r="AA11" s="53"/>
-      <c r="AB11" s="53"/>
+      <c r="A11" s="29"/>
+      <c r="B11" s="29"/>
+      <c r="C11" s="29"/>
+      <c r="D11" s="29"/>
+      <c r="E11" s="29"/>
+      <c r="F11" s="29"/>
+      <c r="G11" s="29"/>
+      <c r="H11" s="30"/>
+      <c r="I11" s="29"/>
+      <c r="J11" s="30"/>
+      <c r="K11" s="31"/>
+      <c r="L11" s="32"/>
+      <c r="M11" s="29"/>
+      <c r="N11" s="29"/>
+      <c r="O11" s="29"/>
+      <c r="P11" s="29"/>
+      <c r="Q11" s="33"/>
+      <c r="R11" s="33"/>
+      <c r="S11" s="33"/>
+      <c r="T11" s="33"/>
+      <c r="U11" s="33"/>
+      <c r="V11" s="33"/>
+      <c r="W11" s="33"/>
+      <c r="X11" s="33"/>
+      <c r="Y11" s="33"/>
+      <c r="Z11" s="26"/>
+      <c r="AA11" s="26"/>
+      <c r="AB11" s="26"/>
     </row>
     <row r="12" spans="1:28" ht="48" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="73"/>
-      <c r="B12" s="73"/>
-      <c r="C12" s="73"/>
-      <c r="D12" s="73"/>
-      <c r="E12" s="73"/>
-      <c r="F12" s="73"/>
-      <c r="G12" s="73"/>
-      <c r="H12" s="74"/>
-      <c r="I12" s="73"/>
-      <c r="J12" s="74"/>
-      <c r="K12" s="75"/>
-      <c r="L12" s="76"/>
-      <c r="M12" s="73"/>
-      <c r="N12" s="73"/>
-      <c r="O12" s="73"/>
-      <c r="P12" s="73"/>
-      <c r="Q12" s="77"/>
-      <c r="R12" s="77"/>
-      <c r="S12" s="77"/>
-      <c r="T12" s="77"/>
-      <c r="U12" s="77"/>
-      <c r="V12" s="77"/>
-      <c r="W12" s="77"/>
-      <c r="X12" s="77"/>
-      <c r="Y12" s="77"/>
-      <c r="Z12" s="53"/>
-      <c r="AA12" s="53"/>
-      <c r="AB12" s="53"/>
+      <c r="A12" s="29"/>
+      <c r="B12" s="29"/>
+      <c r="C12" s="29"/>
+      <c r="D12" s="29"/>
+      <c r="E12" s="29"/>
+      <c r="F12" s="29"/>
+      <c r="G12" s="29"/>
+      <c r="H12" s="30"/>
+      <c r="I12" s="29"/>
+      <c r="J12" s="30"/>
+      <c r="K12" s="31"/>
+      <c r="L12" s="32"/>
+      <c r="M12" s="29"/>
+      <c r="N12" s="29"/>
+      <c r="O12" s="29"/>
+      <c r="P12" s="29"/>
+      <c r="Q12" s="33"/>
+      <c r="R12" s="33"/>
+      <c r="S12" s="33"/>
+      <c r="T12" s="33"/>
+      <c r="U12" s="33"/>
+      <c r="V12" s="33"/>
+      <c r="W12" s="33"/>
+      <c r="X12" s="33"/>
+      <c r="Y12" s="33"/>
+      <c r="Z12" s="26"/>
+      <c r="AA12" s="26"/>
+      <c r="AB12" s="26"/>
     </row>
     <row r="13" spans="1:28" ht="48" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="73"/>
-      <c r="B13" s="73"/>
-      <c r="C13" s="73"/>
-      <c r="D13" s="73"/>
-      <c r="E13" s="73"/>
-      <c r="F13" s="73"/>
-      <c r="G13" s="73"/>
-      <c r="H13" s="74"/>
-      <c r="I13" s="73"/>
-      <c r="J13" s="74"/>
-      <c r="K13" s="75"/>
-      <c r="L13" s="73"/>
-      <c r="M13" s="73"/>
-      <c r="N13" s="73"/>
-      <c r="O13" s="73"/>
-      <c r="P13" s="73"/>
-      <c r="Q13" s="77"/>
-      <c r="R13" s="77"/>
-      <c r="S13" s="77"/>
-      <c r="T13" s="77"/>
-      <c r="U13" s="77"/>
-      <c r="V13" s="77"/>
-      <c r="W13" s="77"/>
-      <c r="X13" s="77"/>
-      <c r="Y13" s="77"/>
-      <c r="Z13" s="53"/>
-      <c r="AA13" s="53"/>
-      <c r="AB13" s="53"/>
+      <c r="A13" s="29"/>
+      <c r="B13" s="29"/>
+      <c r="C13" s="29"/>
+      <c r="D13" s="29"/>
+      <c r="E13" s="29"/>
+      <c r="F13" s="29"/>
+      <c r="G13" s="29"/>
+      <c r="H13" s="30"/>
+      <c r="I13" s="29"/>
+      <c r="J13" s="30"/>
+      <c r="K13" s="31"/>
+      <c r="L13" s="29"/>
+      <c r="M13" s="29"/>
+      <c r="N13" s="29"/>
+      <c r="O13" s="29"/>
+      <c r="P13" s="29"/>
+      <c r="Q13" s="33"/>
+      <c r="R13" s="33"/>
+      <c r="S13" s="33"/>
+      <c r="T13" s="33"/>
+      <c r="U13" s="33"/>
+      <c r="V13" s="33"/>
+      <c r="W13" s="33"/>
+      <c r="X13" s="33"/>
+      <c r="Y13" s="33"/>
+      <c r="Z13" s="26"/>
+      <c r="AA13" s="26"/>
+      <c r="AB13" s="26"/>
     </row>
     <row r="14" spans="1:28" ht="48" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="73"/>
-      <c r="B14" s="73"/>
-      <c r="C14" s="73"/>
-      <c r="D14" s="73"/>
-      <c r="E14" s="73"/>
-      <c r="F14" s="73"/>
-      <c r="G14" s="73"/>
-      <c r="H14" s="74"/>
-      <c r="I14" s="73"/>
-      <c r="J14" s="74"/>
-      <c r="K14" s="75"/>
-      <c r="L14" s="76"/>
-      <c r="M14" s="73"/>
-      <c r="N14" s="73"/>
-      <c r="O14" s="73"/>
-      <c r="P14" s="73"/>
-      <c r="Q14" s="77"/>
-      <c r="R14" s="77"/>
-      <c r="S14" s="77"/>
-      <c r="T14" s="77"/>
-      <c r="U14" s="77"/>
-      <c r="V14" s="77"/>
-      <c r="W14" s="77"/>
-      <c r="X14" s="77"/>
-      <c r="Y14" s="77"/>
-      <c r="Z14" s="53"/>
-      <c r="AA14" s="53"/>
-      <c r="AB14" s="53"/>
+      <c r="A14" s="29"/>
+      <c r="B14" s="29"/>
+      <c r="C14" s="29"/>
+      <c r="D14" s="29"/>
+      <c r="E14" s="29"/>
+      <c r="F14" s="29"/>
+      <c r="G14" s="29"/>
+      <c r="H14" s="30"/>
+      <c r="I14" s="29"/>
+      <c r="J14" s="30"/>
+      <c r="K14" s="31"/>
+      <c r="L14" s="32"/>
+      <c r="M14" s="29"/>
+      <c r="N14" s="29"/>
+      <c r="O14" s="29"/>
+      <c r="P14" s="29"/>
+      <c r="Q14" s="33"/>
+      <c r="R14" s="33"/>
+      <c r="S14" s="33"/>
+      <c r="T14" s="33"/>
+      <c r="U14" s="33"/>
+      <c r="V14" s="33"/>
+      <c r="W14" s="33"/>
+      <c r="X14" s="33"/>
+      <c r="Y14" s="33"/>
+      <c r="Z14" s="26"/>
+      <c r="AA14" s="26"/>
+      <c r="AB14" s="26"/>
     </row>
     <row r="15" spans="1:28" ht="48" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="73"/>
-      <c r="B15" s="73"/>
-      <c r="C15" s="73"/>
-      <c r="D15" s="73"/>
-      <c r="E15" s="73"/>
-      <c r="F15" s="73"/>
-      <c r="G15" s="73"/>
-      <c r="H15" s="74"/>
-      <c r="I15" s="73"/>
-      <c r="J15" s="74"/>
-      <c r="K15" s="75"/>
-      <c r="L15" s="76"/>
-      <c r="M15" s="73"/>
-      <c r="N15" s="73"/>
-      <c r="O15" s="73"/>
-      <c r="P15" s="73"/>
-      <c r="Q15" s="77"/>
-      <c r="R15" s="77"/>
-      <c r="S15" s="77"/>
-      <c r="T15" s="96"/>
-      <c r="U15" s="77"/>
-      <c r="V15" s="77"/>
-      <c r="W15" s="77"/>
-      <c r="X15" s="77"/>
-      <c r="Y15" s="77"/>
-      <c r="Z15" s="53"/>
-      <c r="AA15" s="53"/>
-      <c r="AB15" s="53"/>
+      <c r="A15" s="29"/>
+      <c r="B15" s="29"/>
+      <c r="C15" s="29"/>
+      <c r="D15" s="29"/>
+      <c r="E15" s="29"/>
+      <c r="F15" s="29"/>
+      <c r="G15" s="29"/>
+      <c r="H15" s="30"/>
+      <c r="I15" s="29"/>
+      <c r="J15" s="30"/>
+      <c r="K15" s="31"/>
+      <c r="L15" s="32"/>
+      <c r="M15" s="29"/>
+      <c r="N15" s="29"/>
+      <c r="O15" s="29"/>
+      <c r="P15" s="29"/>
+      <c r="Q15" s="33"/>
+      <c r="R15" s="33"/>
+      <c r="S15" s="33"/>
+      <c r="T15" s="49"/>
+      <c r="U15" s="33"/>
+      <c r="V15" s="33"/>
+      <c r="W15" s="33"/>
+      <c r="X15" s="33"/>
+      <c r="Y15" s="33"/>
+      <c r="Z15" s="26"/>
+      <c r="AA15" s="26"/>
+      <c r="AB15" s="26"/>
     </row>
     <row r="16" spans="1:28" ht="26.25" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A16" s="53"/>
-      <c r="B16" s="53"/>
-      <c r="C16" s="53"/>
-      <c r="D16" s="53"/>
-      <c r="E16" s="53"/>
-      <c r="F16" s="53"/>
-      <c r="G16" s="53"/>
-      <c r="H16" s="53"/>
-      <c r="I16" s="53"/>
-      <c r="J16" s="53"/>
-      <c r="K16" s="53"/>
-      <c r="L16" s="53"/>
-      <c r="M16" s="53"/>
-      <c r="N16" s="53"/>
-      <c r="O16" s="53"/>
-      <c r="P16" s="53"/>
-      <c r="Q16" s="78"/>
-      <c r="R16" s="78"/>
-      <c r="S16" s="78"/>
-      <c r="T16" s="78"/>
-      <c r="U16" s="78"/>
-      <c r="V16" s="78"/>
-      <c r="W16" s="78"/>
-      <c r="X16" s="78"/>
-      <c r="Y16" s="78"/>
-      <c r="Z16" s="53"/>
-      <c r="AA16" s="53"/>
-      <c r="AB16" s="53"/>
+      <c r="A16" s="26"/>
+      <c r="B16" s="26"/>
+      <c r="C16" s="26"/>
+      <c r="D16" s="26"/>
+      <c r="E16" s="26"/>
+      <c r="F16" s="26"/>
+      <c r="G16" s="26"/>
+      <c r="H16" s="26"/>
+      <c r="I16" s="26"/>
+      <c r="J16" s="26"/>
+      <c r="K16" s="26"/>
+      <c r="L16" s="26"/>
+      <c r="M16" s="26"/>
+      <c r="N16" s="26"/>
+      <c r="O16" s="26"/>
+      <c r="P16" s="26"/>
+      <c r="Q16" s="34"/>
+      <c r="R16" s="34"/>
+      <c r="S16" s="34"/>
+      <c r="T16" s="34"/>
+      <c r="U16" s="34"/>
+      <c r="V16" s="34"/>
+      <c r="W16" s="34"/>
+      <c r="X16" s="34"/>
+      <c r="Y16" s="34"/>
+      <c r="Z16" s="26"/>
+      <c r="AA16" s="26"/>
+      <c r="AB16" s="26"/>
     </row>
     <row r="17" spans="1:28" ht="26.25" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A17" s="79"/>
-      <c r="B17" s="53"/>
-      <c r="C17" s="53"/>
-      <c r="D17" s="53"/>
-      <c r="E17" s="53"/>
-      <c r="F17" s="53"/>
-      <c r="G17" s="53"/>
-      <c r="H17" s="53"/>
-      <c r="I17" s="53"/>
-      <c r="J17" s="53"/>
-      <c r="K17" s="80"/>
-      <c r="L17" s="80"/>
-      <c r="M17" s="80"/>
-      <c r="N17" s="80"/>
-      <c r="O17" s="81" t="s">
+      <c r="A17" s="35"/>
+      <c r="B17" s="26"/>
+      <c r="C17" s="26"/>
+      <c r="D17" s="26"/>
+      <c r="E17" s="26"/>
+      <c r="F17" s="26"/>
+      <c r="G17" s="26"/>
+      <c r="H17" s="26"/>
+      <c r="I17" s="26"/>
+      <c r="J17" s="26"/>
+      <c r="K17" s="36"/>
+      <c r="L17" s="36"/>
+      <c r="M17" s="36"/>
+      <c r="N17" s="36"/>
+      <c r="O17" s="50" t="s">
         <v>44</v>
       </c>
-      <c r="P17" s="82"/>
-      <c r="Q17" s="83">
-        <f>SUM(Q11:Q15)</f>
-        <v>0</v>
-      </c>
-      <c r="R17" s="83">
-        <f t="shared" ref="R17:Y17" si="0">SUM(R11:R15)</f>
-        <v>0</v>
-      </c>
-      <c r="S17" s="83">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="T17" s="83">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="U17" s="83">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="V17" s="83">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="W17" s="83">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="X17" s="83">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="Y17" s="83">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="Z17" s="53"/>
-      <c r="AA17" s="53"/>
-      <c r="AB17" s="53"/>
+      <c r="P17" s="51"/>
+      <c r="Q17" s="37"/>
+      <c r="R17" s="37"/>
+      <c r="S17" s="37"/>
+      <c r="T17" s="37"/>
+      <c r="U17" s="37"/>
+      <c r="V17" s="37"/>
+      <c r="W17" s="37"/>
+      <c r="X17" s="37"/>
+      <c r="Y17" s="37"/>
+      <c r="Z17" s="26"/>
+      <c r="AA17" s="26"/>
+      <c r="AB17" s="26"/>
     </row>
     <row r="18" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A18" s="53"/>
-      <c r="B18" s="53"/>
-      <c r="C18" s="53"/>
-      <c r="D18" s="53"/>
-      <c r="E18" s="53"/>
-      <c r="F18" s="53"/>
-      <c r="G18" s="53"/>
-      <c r="H18" s="53"/>
-      <c r="I18" s="53"/>
-      <c r="J18" s="53"/>
-      <c r="K18" s="53"/>
-      <c r="L18" s="53"/>
-      <c r="M18" s="53"/>
-      <c r="N18" s="53"/>
-      <c r="O18" s="53"/>
-      <c r="P18" s="53"/>
-      <c r="Q18" s="53"/>
-      <c r="R18" s="53"/>
-      <c r="S18" s="53"/>
-      <c r="T18" s="53"/>
-      <c r="U18" s="53"/>
-      <c r="V18" s="53"/>
-      <c r="W18" s="53"/>
-      <c r="X18" s="53"/>
-      <c r="Y18" s="53"/>
-      <c r="Z18" s="53"/>
-      <c r="AA18" s="53"/>
-      <c r="AB18" s="53"/>
+      <c r="A18" s="26"/>
+      <c r="B18" s="26"/>
+      <c r="C18" s="26"/>
+      <c r="D18" s="26"/>
+      <c r="E18" s="26"/>
+      <c r="F18" s="26"/>
+      <c r="G18" s="26"/>
+      <c r="H18" s="26"/>
+      <c r="I18" s="26"/>
+      <c r="J18" s="26"/>
+      <c r="K18" s="26"/>
+      <c r="L18" s="26"/>
+      <c r="M18" s="26"/>
+      <c r="N18" s="26"/>
+      <c r="O18" s="26"/>
+      <c r="P18" s="26"/>
+      <c r="Q18" s="26"/>
+      <c r="R18" s="26"/>
+      <c r="S18" s="26"/>
+      <c r="T18" s="26"/>
+      <c r="U18" s="26"/>
+      <c r="V18" s="26"/>
+      <c r="W18" s="26"/>
+      <c r="X18" s="26"/>
+      <c r="Y18" s="26"/>
+      <c r="Z18" s="26"/>
+      <c r="AA18" s="26"/>
+      <c r="AB18" s="26"/>
     </row>
     <row r="19" spans="1:28" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A19" s="84" t="s">
+      <c r="A19" s="38" t="s">
         <v>45</v>
       </c>
-      <c r="B19" s="85"/>
-      <c r="C19" s="86"/>
-      <c r="D19" s="53"/>
-      <c r="E19" s="53"/>
-      <c r="F19" s="53"/>
-      <c r="G19" s="53"/>
-      <c r="H19" s="53"/>
-      <c r="I19" s="53"/>
-      <c r="J19" s="53"/>
-      <c r="K19" s="53"/>
-      <c r="L19" s="53"/>
-      <c r="M19" s="53"/>
-      <c r="N19" s="53"/>
-      <c r="O19" s="53"/>
-      <c r="P19" s="53"/>
-      <c r="Q19" s="53"/>
-      <c r="R19" s="53"/>
-      <c r="S19" s="87"/>
-      <c r="T19" s="88"/>
-      <c r="U19" s="88"/>
-      <c r="V19" s="88"/>
-      <c r="W19" s="88"/>
-      <c r="X19" s="88"/>
-      <c r="Y19" s="89"/>
-      <c r="Z19" s="53"/>
-      <c r="AA19" s="53"/>
-      <c r="AB19" s="53"/>
+      <c r="B19" s="39"/>
+      <c r="C19" s="40"/>
+      <c r="D19" s="26"/>
+      <c r="E19" s="26"/>
+      <c r="F19" s="26"/>
+      <c r="G19" s="26"/>
+      <c r="H19" s="26"/>
+      <c r="I19" s="26"/>
+      <c r="J19" s="26"/>
+      <c r="K19" s="26"/>
+      <c r="L19" s="26"/>
+      <c r="M19" s="26"/>
+      <c r="N19" s="26"/>
+      <c r="O19" s="26"/>
+      <c r="P19" s="26"/>
+      <c r="Q19" s="26"/>
+      <c r="R19" s="26"/>
+      <c r="S19" s="41"/>
+      <c r="T19" s="42"/>
+      <c r="U19" s="42"/>
+      <c r="V19" s="42"/>
+      <c r="W19" s="42"/>
+      <c r="X19" s="42"/>
+      <c r="Y19" s="43"/>
+      <c r="Z19" s="26"/>
+      <c r="AA19" s="26"/>
+      <c r="AB19" s="26"/>
     </row>
     <row r="20" spans="1:28" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A20" s="85"/>
-      <c r="B20" s="85"/>
-      <c r="C20" s="86"/>
-      <c r="D20" s="53"/>
-      <c r="E20" s="53"/>
-      <c r="F20" s="53"/>
-      <c r="G20" s="53"/>
-      <c r="H20" s="53"/>
-      <c r="I20" s="53"/>
-      <c r="J20" s="53"/>
-      <c r="K20" s="53"/>
-      <c r="L20" s="53"/>
-      <c r="M20" s="53"/>
-      <c r="N20" s="53"/>
-      <c r="O20" s="53"/>
-      <c r="P20" s="53"/>
-      <c r="Q20" s="79"/>
-      <c r="R20" s="79"/>
-      <c r="S20" s="87"/>
-      <c r="T20" s="88"/>
-      <c r="U20" s="88"/>
-      <c r="V20" s="88"/>
-      <c r="W20" s="88"/>
-      <c r="X20" s="88"/>
-      <c r="Y20" s="89"/>
-      <c r="Z20" s="53"/>
-      <c r="AA20" s="53"/>
-      <c r="AB20" s="53"/>
+      <c r="A20" s="39"/>
+      <c r="B20" s="39"/>
+      <c r="C20" s="40"/>
+      <c r="D20" s="26"/>
+      <c r="E20" s="26"/>
+      <c r="F20" s="26"/>
+      <c r="G20" s="26"/>
+      <c r="H20" s="26"/>
+      <c r="I20" s="26"/>
+      <c r="J20" s="26"/>
+      <c r="K20" s="26"/>
+      <c r="L20" s="26"/>
+      <c r="M20" s="26"/>
+      <c r="N20" s="26"/>
+      <c r="O20" s="26"/>
+      <c r="P20" s="26"/>
+      <c r="Q20" s="35"/>
+      <c r="R20" s="35"/>
+      <c r="S20" s="41"/>
+      <c r="T20" s="42"/>
+      <c r="U20" s="42"/>
+      <c r="V20" s="42"/>
+      <c r="W20" s="42"/>
+      <c r="X20" s="42"/>
+      <c r="Y20" s="43"/>
+      <c r="Z20" s="26"/>
+      <c r="AA20" s="26"/>
+      <c r="AB20" s="26"/>
     </row>
     <row r="21" spans="1:28" ht="20.25" x14ac:dyDescent="0.3">
-      <c r="A21" s="90" t="s">
+      <c r="A21" s="44" t="s">
         <v>46</v>
       </c>
-      <c r="B21" s="85"/>
-      <c r="C21" s="86"/>
-      <c r="D21" s="53"/>
-      <c r="E21" s="53"/>
-      <c r="F21" s="53"/>
-      <c r="G21" s="91" t="s">
+      <c r="B21" s="39"/>
+      <c r="C21" s="40"/>
+      <c r="D21" s="26"/>
+      <c r="E21" s="26"/>
+      <c r="F21" s="26"/>
+      <c r="G21" s="52" t="s">
         <v>47</v>
       </c>
-      <c r="H21" s="91"/>
-      <c r="I21" s="53"/>
-      <c r="J21" s="53"/>
-      <c r="K21" s="53"/>
-      <c r="L21" s="92"/>
-      <c r="M21" s="91" t="s">
+      <c r="H21" s="52"/>
+      <c r="I21" s="26"/>
+      <c r="J21" s="26"/>
+      <c r="K21" s="26"/>
+      <c r="L21" s="45"/>
+      <c r="M21" s="52" t="s">
         <v>48</v>
       </c>
-      <c r="N21" s="91"/>
-      <c r="O21" s="53"/>
-      <c r="P21" s="53"/>
-      <c r="Q21" s="53"/>
-      <c r="R21" s="53"/>
-      <c r="S21" s="87"/>
-      <c r="T21" s="88"/>
-      <c r="U21" s="88"/>
-      <c r="V21" s="88"/>
-      <c r="W21" s="88"/>
-      <c r="X21" s="88"/>
-      <c r="Y21" s="89"/>
-      <c r="Z21" s="53"/>
-      <c r="AA21" s="53"/>
-      <c r="AB21" s="53"/>
+      <c r="N21" s="52"/>
+      <c r="O21" s="26"/>
+      <c r="P21" s="26"/>
+      <c r="Q21" s="26"/>
+      <c r="R21" s="26"/>
+      <c r="S21" s="41"/>
+      <c r="T21" s="42"/>
+      <c r="U21" s="42"/>
+      <c r="V21" s="42"/>
+      <c r="W21" s="42"/>
+      <c r="X21" s="42"/>
+      <c r="Y21" s="43"/>
+      <c r="Z21" s="26"/>
+      <c r="AA21" s="26"/>
+      <c r="AB21" s="26"/>
     </row>
     <row r="22" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A22" s="85"/>
-      <c r="B22" s="85"/>
-      <c r="C22" s="86"/>
-      <c r="D22" s="53"/>
-      <c r="O22" s="53"/>
-      <c r="P22" s="53"/>
-      <c r="S22" s="53"/>
-      <c r="T22" s="53"/>
-      <c r="U22" s="53"/>
-      <c r="V22" s="53"/>
-      <c r="W22" s="53"/>
-      <c r="X22" s="53"/>
-      <c r="Y22" s="53"/>
-      <c r="Z22" s="53"/>
-      <c r="AA22" s="53"/>
-      <c r="AB22" s="53"/>
+      <c r="A22" s="39"/>
+      <c r="B22" s="39"/>
+      <c r="C22" s="40"/>
+      <c r="D22" s="26"/>
+      <c r="O22" s="26"/>
+      <c r="P22" s="26"/>
+      <c r="S22" s="26"/>
+      <c r="T22" s="26"/>
+      <c r="U22" s="26"/>
+      <c r="V22" s="26"/>
+      <c r="W22" s="26"/>
+      <c r="X22" s="26"/>
+      <c r="Y22" s="26"/>
+      <c r="Z22" s="26"/>
+      <c r="AA22" s="26"/>
+      <c r="AB22" s="26"/>
     </row>
     <row r="23" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A23" s="90" t="str">
+      <c r="A23" s="44" t="str">
         <f>+'[1]ANEXO NP1'!A78</f>
         <v>MES: FEBRERO   AÑO: 2025</v>
       </c>
-      <c r="B23" s="85"/>
-      <c r="C23" s="86"/>
-      <c r="D23" s="53"/>
-      <c r="E23" s="53"/>
-      <c r="F23" s="53"/>
-      <c r="G23" s="53"/>
-      <c r="H23" s="53"/>
-      <c r="I23" s="53"/>
-      <c r="J23" s="53"/>
-      <c r="K23" s="93"/>
-      <c r="L23" s="53"/>
-      <c r="M23" s="93"/>
+      <c r="B23" s="39"/>
+      <c r="C23" s="40"/>
+      <c r="D23" s="26"/>
+      <c r="E23" s="26"/>
+      <c r="F23" s="26"/>
+      <c r="G23" s="26"/>
+      <c r="H23" s="26"/>
+      <c r="I23" s="26"/>
+      <c r="J23" s="26"/>
+      <c r="K23" s="46"/>
+      <c r="L23" s="26"/>
+      <c r="M23" s="46"/>
       <c r="N23" s="1"/>
-      <c r="O23" s="93"/>
-      <c r="P23" s="53"/>
-      <c r="S23" s="53"/>
+      <c r="O23" s="46"/>
+      <c r="P23" s="26"/>
+      <c r="S23" s="26"/>
       <c r="T23" s="1"/>
       <c r="U23" s="1"/>
       <c r="V23" s="1"/>
       <c r="W23" s="1"/>
       <c r="X23" s="1"/>
-      <c r="Y23" s="53"/>
-      <c r="Z23" s="53"/>
-      <c r="AA23" s="53"/>
-      <c r="AB23" s="53"/>
+      <c r="Y23" s="26"/>
+      <c r="Z23" s="26"/>
+      <c r="AA23" s="26"/>
+      <c r="AB23" s="26"/>
     </row>
     <row r="24" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A24" s="1"/>
-      <c r="B24" s="53"/>
-      <c r="K24" s="53"/>
-      <c r="L24" s="53"/>
-      <c r="M24" s="53"/>
-      <c r="N24" s="53"/>
-      <c r="O24" s="53"/>
-      <c r="P24" s="53"/>
-      <c r="S24" s="53"/>
-      <c r="T24" s="53"/>
-      <c r="U24" s="53"/>
-      <c r="V24" s="53"/>
-      <c r="W24" s="53"/>
-      <c r="X24" s="53"/>
-      <c r="Y24" s="53"/>
-      <c r="Z24" s="53"/>
-      <c r="AA24" s="53"/>
-      <c r="AB24" s="53"/>
+      <c r="B24" s="26"/>
+      <c r="K24" s="26"/>
+      <c r="L24" s="26"/>
+      <c r="M24" s="26"/>
+      <c r="N24" s="26"/>
+      <c r="O24" s="26"/>
+      <c r="P24" s="26"/>
+      <c r="S24" s="26"/>
+      <c r="T24" s="26"/>
+      <c r="U24" s="26"/>
+      <c r="V24" s="26"/>
+      <c r="W24" s="26"/>
+      <c r="X24" s="26"/>
+      <c r="Y24" s="26"/>
+      <c r="Z24" s="26"/>
+      <c r="AA24" s="26"/>
+      <c r="AB24" s="26"/>
     </row>
     <row r="25" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A25" s="1"/>
-      <c r="B25" s="53"/>
-      <c r="C25" s="53"/>
-      <c r="D25" s="53"/>
-      <c r="E25" s="53"/>
-      <c r="F25" s="53"/>
-      <c r="G25" s="53"/>
-      <c r="H25" s="53"/>
-      <c r="I25" s="53"/>
-      <c r="J25" s="53"/>
-      <c r="K25" s="53"/>
-      <c r="L25" s="53"/>
-      <c r="M25" s="53"/>
-      <c r="N25" s="53"/>
-      <c r="O25" s="53"/>
-      <c r="P25" s="53"/>
-      <c r="Q25" s="53"/>
-      <c r="R25" s="53"/>
-      <c r="S25" s="53"/>
-      <c r="T25" s="53"/>
-      <c r="U25" s="53"/>
-      <c r="V25" s="53"/>
-      <c r="W25" s="53"/>
-      <c r="X25" s="53"/>
-      <c r="Y25" s="94" t="s">
+      <c r="B25" s="26"/>
+      <c r="C25" s="26"/>
+      <c r="D25" s="26"/>
+      <c r="E25" s="26"/>
+      <c r="F25" s="26"/>
+      <c r="G25" s="26"/>
+      <c r="H25" s="26"/>
+      <c r="I25" s="26"/>
+      <c r="J25" s="26"/>
+      <c r="K25" s="26"/>
+      <c r="L25" s="26"/>
+      <c r="M25" s="26"/>
+      <c r="N25" s="26"/>
+      <c r="O25" s="26"/>
+      <c r="P25" s="26"/>
+      <c r="Q25" s="26"/>
+      <c r="R25" s="26"/>
+      <c r="S25" s="26"/>
+      <c r="T25" s="26"/>
+      <c r="U25" s="26"/>
+      <c r="V25" s="26"/>
+      <c r="W25" s="26"/>
+      <c r="X25" s="26"/>
+      <c r="Y25" s="47" t="s">
         <v>49</v>
       </c>
-      <c r="Z25" s="53"/>
-      <c r="AA25" s="53"/>
-      <c r="AB25" s="53"/>
+      <c r="Z25" s="26"/>
+      <c r="AA25" s="26"/>
+      <c r="AB25" s="26"/>
     </row>
     <row r="26" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A26" s="79"/>
-      <c r="B26" s="53"/>
-      <c r="C26" s="53"/>
-      <c r="D26" s="53"/>
-      <c r="E26" s="53"/>
-      <c r="F26" s="53"/>
-      <c r="G26" s="53"/>
-      <c r="H26" s="53"/>
-      <c r="I26" s="53"/>
-      <c r="J26" s="53"/>
-      <c r="K26" s="53"/>
-      <c r="L26" s="53"/>
-      <c r="M26" s="53"/>
-      <c r="N26" s="53"/>
-      <c r="O26" s="53"/>
-      <c r="P26" s="53"/>
-      <c r="Q26" s="53"/>
-      <c r="R26" s="53"/>
-      <c r="S26" s="53"/>
-      <c r="T26" s="53"/>
-      <c r="U26" s="53"/>
-      <c r="V26" s="53"/>
-      <c r="W26" s="53"/>
-      <c r="X26" s="53"/>
-      <c r="Y26" s="53"/>
-      <c r="Z26" s="53"/>
-      <c r="AA26" s="53"/>
-      <c r="AB26" s="53"/>
+      <c r="A26" s="35"/>
+      <c r="B26" s="26"/>
+      <c r="C26" s="26"/>
+      <c r="D26" s="26"/>
+      <c r="E26" s="26"/>
+      <c r="F26" s="26"/>
+      <c r="G26" s="26"/>
+      <c r="H26" s="26"/>
+      <c r="I26" s="26"/>
+      <c r="J26" s="26"/>
+      <c r="K26" s="26"/>
+      <c r="L26" s="26"/>
+      <c r="M26" s="26"/>
+      <c r="N26" s="26"/>
+      <c r="O26" s="26"/>
+      <c r="P26" s="26"/>
+      <c r="Q26" s="26"/>
+      <c r="R26" s="26"/>
+      <c r="S26" s="26"/>
+      <c r="T26" s="26"/>
+      <c r="U26" s="26"/>
+      <c r="V26" s="26"/>
+      <c r="W26" s="26"/>
+      <c r="X26" s="26"/>
+      <c r="Y26" s="26"/>
+      <c r="Z26" s="26"/>
+      <c r="AA26" s="26"/>
+      <c r="AB26" s="26"/>
     </row>
     <row r="27" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A27" s="53"/>
-      <c r="B27" s="53"/>
-      <c r="C27" s="53"/>
-      <c r="D27" s="53"/>
-      <c r="E27" s="53"/>
-      <c r="F27" s="53"/>
-      <c r="G27" s="53"/>
-      <c r="H27" s="53"/>
-      <c r="I27" s="53"/>
-      <c r="J27" s="53"/>
-      <c r="K27" s="53"/>
-      <c r="L27" s="53"/>
-      <c r="M27" s="53"/>
-      <c r="N27" s="53"/>
-      <c r="O27" s="53"/>
-      <c r="P27" s="53"/>
-      <c r="Q27" s="53"/>
-      <c r="R27" s="53"/>
-      <c r="S27" s="79"/>
-      <c r="T27" s="53"/>
-      <c r="U27" s="53"/>
-      <c r="V27" s="53"/>
-      <c r="W27" s="53"/>
-      <c r="X27" s="53"/>
-      <c r="Y27" s="53"/>
-      <c r="Z27" s="53"/>
-      <c r="AA27" s="53"/>
-      <c r="AB27" s="53"/>
+      <c r="A27" s="26"/>
+      <c r="B27" s="26"/>
+      <c r="C27" s="26"/>
+      <c r="D27" s="26"/>
+      <c r="E27" s="26"/>
+      <c r="F27" s="26"/>
+      <c r="G27" s="26"/>
+      <c r="H27" s="26"/>
+      <c r="I27" s="26"/>
+      <c r="J27" s="26"/>
+      <c r="K27" s="26"/>
+      <c r="L27" s="26"/>
+      <c r="M27" s="26"/>
+      <c r="N27" s="26"/>
+      <c r="O27" s="26"/>
+      <c r="P27" s="26"/>
+      <c r="Q27" s="26"/>
+      <c r="R27" s="26"/>
+      <c r="S27" s="35"/>
+      <c r="T27" s="26"/>
+      <c r="U27" s="26"/>
+      <c r="V27" s="26"/>
+      <c r="W27" s="26"/>
+      <c r="X27" s="26"/>
+      <c r="Y27" s="26"/>
+      <c r="Z27" s="26"/>
+      <c r="AA27" s="26"/>
+      <c r="AB27" s="26"/>
     </row>
     <row r="28" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A28" s="53"/>
-      <c r="B28" s="53"/>
-      <c r="C28" s="53"/>
-      <c r="D28" s="53"/>
-      <c r="E28" s="53"/>
-      <c r="F28" s="53"/>
-      <c r="G28" s="53"/>
-      <c r="H28" s="53"/>
-      <c r="I28" s="53"/>
-      <c r="J28" s="53"/>
-      <c r="K28" s="53"/>
-      <c r="L28" s="53"/>
-      <c r="M28" s="53"/>
-      <c r="N28" s="53"/>
-      <c r="O28" s="53"/>
-      <c r="P28" s="53"/>
-      <c r="Q28" s="53"/>
-      <c r="R28" s="53"/>
-      <c r="S28" s="53"/>
-      <c r="T28" s="53"/>
-      <c r="U28" s="53"/>
-      <c r="V28" s="53"/>
-      <c r="W28" s="53"/>
-      <c r="X28" s="53"/>
-      <c r="Y28" s="53"/>
-      <c r="Z28" s="53"/>
-      <c r="AA28" s="53"/>
-      <c r="AB28" s="53"/>
+      <c r="A28" s="26"/>
+      <c r="B28" s="26"/>
+      <c r="C28" s="26"/>
+      <c r="D28" s="26"/>
+      <c r="E28" s="26"/>
+      <c r="F28" s="26"/>
+      <c r="G28" s="26"/>
+      <c r="H28" s="26"/>
+      <c r="I28" s="26"/>
+      <c r="J28" s="26"/>
+      <c r="K28" s="26"/>
+      <c r="L28" s="26"/>
+      <c r="M28" s="26"/>
+      <c r="N28" s="26"/>
+      <c r="O28" s="26"/>
+      <c r="P28" s="26"/>
+      <c r="Q28" s="26"/>
+      <c r="R28" s="26"/>
+      <c r="S28" s="26"/>
+      <c r="T28" s="26"/>
+      <c r="U28" s="26"/>
+      <c r="V28" s="26"/>
+      <c r="W28" s="26"/>
+      <c r="X28" s="26"/>
+      <c r="Y28" s="26"/>
+      <c r="Z28" s="26"/>
+      <c r="AA28" s="26"/>
+      <c r="AB28" s="26"/>
     </row>
     <row r="29" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A29" s="53"/>
-      <c r="B29" s="53"/>
-      <c r="C29" s="53"/>
-      <c r="D29" s="53"/>
-      <c r="E29" s="53"/>
-      <c r="F29" s="53"/>
-      <c r="G29" s="53"/>
-      <c r="H29" s="53"/>
-      <c r="I29" s="53"/>
-      <c r="J29" s="53"/>
-      <c r="K29" s="53"/>
-      <c r="L29" s="53"/>
-      <c r="M29" s="53"/>
-      <c r="N29" s="53"/>
-      <c r="O29" s="53"/>
-      <c r="P29" s="53"/>
-      <c r="Q29" s="53"/>
-      <c r="R29" s="53"/>
-      <c r="S29" s="53"/>
-      <c r="T29" s="53"/>
-      <c r="U29" s="53"/>
-      <c r="V29" s="53"/>
-      <c r="W29" s="53"/>
-      <c r="X29" s="53"/>
-      <c r="Y29" s="53"/>
-      <c r="Z29" s="53"/>
-      <c r="AA29" s="95"/>
-      <c r="AB29" s="53"/>
+      <c r="A29" s="26"/>
+      <c r="B29" s="26"/>
+      <c r="C29" s="26"/>
+      <c r="D29" s="26"/>
+      <c r="E29" s="26"/>
+      <c r="F29" s="26"/>
+      <c r="G29" s="26"/>
+      <c r="H29" s="26"/>
+      <c r="I29" s="26"/>
+      <c r="J29" s="26"/>
+      <c r="K29" s="26"/>
+      <c r="L29" s="26"/>
+      <c r="M29" s="26"/>
+      <c r="N29" s="26"/>
+      <c r="O29" s="26"/>
+      <c r="P29" s="26"/>
+      <c r="Q29" s="26"/>
+      <c r="R29" s="26"/>
+      <c r="S29" s="26"/>
+      <c r="T29" s="26"/>
+      <c r="U29" s="26"/>
+      <c r="V29" s="26"/>
+      <c r="W29" s="26"/>
+      <c r="X29" s="26"/>
+      <c r="Y29" s="26"/>
+      <c r="Z29" s="26"/>
+      <c r="AA29" s="48"/>
+      <c r="AB29" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="33">
-    <mergeCell ref="O17:P17"/>
-    <mergeCell ref="G21:H21"/>
-    <mergeCell ref="M21:N21"/>
-    <mergeCell ref="T7:T10"/>
-    <mergeCell ref="U7:U10"/>
+    <mergeCell ref="O2:Y2"/>
+    <mergeCell ref="O3:Y3"/>
+    <mergeCell ref="O4:Y4"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="K6:O6"/>
+    <mergeCell ref="A7:A10"/>
+    <mergeCell ref="B7:B10"/>
+    <mergeCell ref="C7:C10"/>
+    <mergeCell ref="D7:D10"/>
+    <mergeCell ref="E7:E10"/>
     <mergeCell ref="V7:V10"/>
     <mergeCell ref="W7:W10"/>
     <mergeCell ref="X7:X10"/>
@@ -3147,20 +3126,14 @@
     <mergeCell ref="I9:I10"/>
     <mergeCell ref="K9:K10"/>
     <mergeCell ref="L9:O9"/>
-    <mergeCell ref="A7:A10"/>
-    <mergeCell ref="B7:B10"/>
-    <mergeCell ref="C7:C10"/>
-    <mergeCell ref="D7:D10"/>
-    <mergeCell ref="E7:E10"/>
+    <mergeCell ref="O17:P17"/>
+    <mergeCell ref="G21:H21"/>
+    <mergeCell ref="M21:N21"/>
+    <mergeCell ref="T7:T10"/>
+    <mergeCell ref="U7:U10"/>
     <mergeCell ref="F7:G8"/>
     <mergeCell ref="F9:F10"/>
     <mergeCell ref="G9:G10"/>
-    <mergeCell ref="O2:Y2"/>
-    <mergeCell ref="O3:Y3"/>
-    <mergeCell ref="O4:Y4"/>
-    <mergeCell ref="F6:G6"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="K6:O6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="35" orientation="landscape" r:id="rId1"/>

</xml_diff>

<commit_message>
Refactor annex payroll generation and add directivo template
Refactors the teachers payroll annex generation to use the 'ANEXO NOMINA DE PAGO PERSONAL DIRECTIVO.xlsx' template, generating separate annex files for each group of professors. Enhances the date-organized path helper to support category and subcategory folders. Updates OpenAPI tags and adds the 'xlsx' dependency. New template file for directivo annex is included.
</commit_message>
<xml_diff>
--- a/src/core/excel/templates/ANEXO NOMINA DE PAGO PERSONAL ADMINISTRATIVO.xlsx
+++ b/src/core/excel/templates/ANEXO NOMINA DE PAGO PERSONAL ADMINISTRATIVO.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\david\OneDrive\Documentos\Codigo\san-miguel-porres-backend\src\core\excel\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0E9D5D8-1D71-4DD6-BD27-F56BF7AEBB8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B46FF5FD-834C-423F-BEE9-AFF08AEC7C41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,6 +20,7 @@
   </externalReferences>
   <definedNames>
     <definedName name="_xlnm.Extract">#REF!</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'ANEXO NP2 A'!$A$1:$AA$45</definedName>
     <definedName name="_xlnm.Database">#REF!</definedName>
     <definedName name="_xlnm.Criteria">#REF!</definedName>
     <definedName name="V">#REF!</definedName>
@@ -201,7 +202,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="17" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -299,6 +300,13 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="18"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -506,7 +514,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="97">
+  <cellXfs count="101">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -599,9 +607,6 @@
     <xf numFmtId="4" fontId="12" fillId="0" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="4" fontId="12" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -645,139 +650,144 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="4" fontId="12" fillId="0" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1034,13 +1044,13 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>200025</xdr:colOff>
-      <xdr:row>19</xdr:row>
+      <xdr:row>32</xdr:row>
       <xdr:rowOff>219075</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>333375</xdr:colOff>
-      <xdr:row>19</xdr:row>
+      <xdr:row>32</xdr:row>
       <xdr:rowOff>219075</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -1152,14 +1162,14 @@
     <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>457200</xdr:colOff>
-      <xdr:row>22</xdr:row>
+      <xdr:row>35</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>19</xdr:col>
       <xdr:colOff>219075</xdr:colOff>
-      <xdr:row>24</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1253,7 +1263,13 @@
       <sheetName val="NP4"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0"/>
+      <sheetData sheetId="0">
+        <row r="1">
+          <cell r="B1" t="str">
+            <v>MES: FEBRERO   AÑO: 2025</v>
+          </cell>
+        </row>
+      </sheetData>
       <sheetData sheetId="1"/>
       <sheetData sheetId="2"/>
       <sheetData sheetId="3">
@@ -1549,7 +1565,7 @@
   <sheetPr>
     <tabColor rgb="FF002060"/>
   </sheetPr>
-  <dimension ref="A1:AB29"/>
+  <dimension ref="A1:AB39"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6.140625" style="3" customWidth="1"/>
@@ -2183,19 +2199,19 @@
       <c r="L2" s="8"/>
       <c r="M2" s="8"/>
       <c r="N2" s="8"/>
-      <c r="O2" s="88" t="s">
+      <c r="O2" s="51" t="s">
         <v>4</v>
       </c>
-      <c r="P2" s="89"/>
-      <c r="Q2" s="89"/>
-      <c r="R2" s="89"/>
-      <c r="S2" s="89"/>
-      <c r="T2" s="89"/>
-      <c r="U2" s="89"/>
-      <c r="V2" s="89"/>
-      <c r="W2" s="89"/>
-      <c r="X2" s="89"/>
-      <c r="Y2" s="90"/>
+      <c r="P2" s="52"/>
+      <c r="Q2" s="52"/>
+      <c r="R2" s="52"/>
+      <c r="S2" s="52"/>
+      <c r="T2" s="52"/>
+      <c r="U2" s="52"/>
+      <c r="V2" s="52"/>
+      <c r="W2" s="52"/>
+      <c r="X2" s="52"/>
+      <c r="Y2" s="53"/>
       <c r="Z2" s="1"/>
       <c r="AA2" s="1"/>
       <c r="AB2" s="1"/>
@@ -2217,19 +2233,19 @@
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
       <c r="N3" s="1"/>
-      <c r="O3" s="91" t="s">
+      <c r="O3" s="98" t="s">
         <v>6</v>
       </c>
-      <c r="P3" s="92"/>
-      <c r="Q3" s="92"/>
-      <c r="R3" s="92"/>
-      <c r="S3" s="92"/>
-      <c r="T3" s="92"/>
-      <c r="U3" s="92"/>
-      <c r="V3" s="92"/>
-      <c r="W3" s="92"/>
-      <c r="X3" s="92"/>
-      <c r="Y3" s="93"/>
+      <c r="P3" s="99"/>
+      <c r="Q3" s="99"/>
+      <c r="R3" s="99"/>
+      <c r="S3" s="99"/>
+      <c r="T3" s="99"/>
+      <c r="U3" s="99"/>
+      <c r="V3" s="99"/>
+      <c r="W3" s="99"/>
+      <c r="X3" s="99"/>
+      <c r="Y3" s="100"/>
       <c r="Z3" s="1"/>
       <c r="AA3" s="1"/>
       <c r="AB3" s="1"/>
@@ -2251,19 +2267,19 @@
       <c r="L4" s="18"/>
       <c r="M4" s="18"/>
       <c r="N4" s="18"/>
-      <c r="O4" s="94" t="s">
+      <c r="O4" s="54" t="s">
         <v>8</v>
       </c>
-      <c r="P4" s="95"/>
-      <c r="Q4" s="95"/>
-      <c r="R4" s="95"/>
-      <c r="S4" s="95"/>
-      <c r="T4" s="95"/>
-      <c r="U4" s="95"/>
-      <c r="V4" s="95"/>
-      <c r="W4" s="95"/>
-      <c r="X4" s="95"/>
-      <c r="Y4" s="96"/>
+      <c r="P4" s="55"/>
+      <c r="Q4" s="55"/>
+      <c r="R4" s="55"/>
+      <c r="S4" s="55"/>
+      <c r="T4" s="55"/>
+      <c r="U4" s="55"/>
+      <c r="V4" s="55"/>
+      <c r="W4" s="55"/>
+      <c r="X4" s="55"/>
+      <c r="Y4" s="56"/>
       <c r="Z4" s="1"/>
       <c r="AA4" s="1"/>
       <c r="AB4" s="1"/>
@@ -2312,24 +2328,24 @@
       <c r="E6" s="23">
         <v>4</v>
       </c>
-      <c r="F6" s="77">
+      <c r="F6" s="57">
         <v>5</v>
       </c>
-      <c r="G6" s="79"/>
-      <c r="H6" s="77">
+      <c r="G6" s="58"/>
+      <c r="H6" s="57">
         <v>6</v>
       </c>
-      <c r="I6" s="79"/>
+      <c r="I6" s="58"/>
       <c r="J6" s="23">
         <v>7</v>
       </c>
-      <c r="K6" s="77">
+      <c r="K6" s="57">
         <v>8</v>
       </c>
-      <c r="L6" s="78"/>
-      <c r="M6" s="78"/>
-      <c r="N6" s="78"/>
-      <c r="O6" s="79"/>
+      <c r="L6" s="59"/>
+      <c r="M6" s="59"/>
+      <c r="N6" s="59"/>
+      <c r="O6" s="58"/>
       <c r="P6" s="23">
         <v>9</v>
       </c>
@@ -2365,63 +2381,63 @@
       <c r="AB6" s="24"/>
     </row>
     <row r="7" spans="1:28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="73" t="s">
+      <c r="A7" s="60" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="80" t="s">
+      <c r="B7" s="62" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="82" t="s">
+      <c r="C7" s="64" t="s">
         <v>19</v>
       </c>
-      <c r="D7" s="82"/>
-      <c r="E7" s="84" t="s">
+      <c r="D7" s="64"/>
+      <c r="E7" s="66" t="s">
         <v>20</v>
       </c>
-      <c r="F7" s="61" t="s">
+      <c r="F7" s="76" t="s">
         <v>21</v>
       </c>
-      <c r="G7" s="86"/>
-      <c r="H7" s="61" t="s">
+      <c r="G7" s="91"/>
+      <c r="H7" s="76" t="s">
         <v>22</v>
       </c>
-      <c r="I7" s="62"/>
-      <c r="J7" s="65" t="s">
+      <c r="I7" s="77"/>
+      <c r="J7" s="80" t="s">
         <v>23</v>
       </c>
-      <c r="K7" s="67" t="s">
+      <c r="K7" s="82" t="s">
         <v>24</v>
       </c>
-      <c r="L7" s="68"/>
-      <c r="M7" s="68"/>
-      <c r="N7" s="68"/>
-      <c r="O7" s="69"/>
+      <c r="L7" s="83"/>
+      <c r="M7" s="83"/>
+      <c r="N7" s="83"/>
+      <c r="O7" s="84"/>
       <c r="P7" s="25"/>
-      <c r="Q7" s="53" t="s">
+      <c r="Q7" s="70" t="s">
         <v>25</v>
       </c>
-      <c r="R7" s="53" t="s">
+      <c r="R7" s="70" t="s">
         <v>26</v>
       </c>
-      <c r="S7" s="53" t="s">
+      <c r="S7" s="70" t="s">
         <v>27</v>
       </c>
-      <c r="T7" s="53" t="s">
+      <c r="T7" s="70" t="s">
         <v>28</v>
       </c>
-      <c r="U7" s="55" t="s">
+      <c r="U7" s="68" t="s">
         <v>29</v>
       </c>
-      <c r="V7" s="55" t="s">
+      <c r="V7" s="68" t="s">
         <v>30</v>
       </c>
-      <c r="W7" s="53" t="s">
+      <c r="W7" s="70" t="s">
         <v>31</v>
       </c>
-      <c r="X7" s="57" t="s">
+      <c r="X7" s="72" t="s">
         <v>32</v>
       </c>
-      <c r="Y7" s="59" t="s">
+      <c r="Y7" s="74" t="s">
         <v>33</v>
       </c>
       <c r="Z7" s="26"/>
@@ -2429,89 +2445,89 @@
       <c r="AB7" s="26"/>
     </row>
     <row r="8" spans="1:28" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="74"/>
-      <c r="B8" s="81"/>
-      <c r="C8" s="83"/>
-      <c r="D8" s="83"/>
-      <c r="E8" s="85"/>
-      <c r="F8" s="63"/>
-      <c r="G8" s="87"/>
-      <c r="H8" s="63"/>
-      <c r="I8" s="64"/>
-      <c r="J8" s="66"/>
-      <c r="K8" s="70"/>
-      <c r="L8" s="71"/>
-      <c r="M8" s="71"/>
-      <c r="N8" s="71"/>
-      <c r="O8" s="72"/>
+      <c r="A8" s="61"/>
+      <c r="B8" s="63"/>
+      <c r="C8" s="65"/>
+      <c r="D8" s="65"/>
+      <c r="E8" s="67"/>
+      <c r="F8" s="78"/>
+      <c r="G8" s="92"/>
+      <c r="H8" s="78"/>
+      <c r="I8" s="79"/>
+      <c r="J8" s="81"/>
+      <c r="K8" s="85"/>
+      <c r="L8" s="86"/>
+      <c r="M8" s="86"/>
+      <c r="N8" s="86"/>
+      <c r="O8" s="87"/>
       <c r="P8" s="27"/>
-      <c r="Q8" s="54"/>
-      <c r="R8" s="54"/>
-      <c r="S8" s="54"/>
-      <c r="T8" s="54"/>
-      <c r="U8" s="56"/>
-      <c r="V8" s="56"/>
-      <c r="W8" s="54"/>
-      <c r="X8" s="58"/>
-      <c r="Y8" s="60"/>
+      <c r="Q8" s="71"/>
+      <c r="R8" s="71"/>
+      <c r="S8" s="71"/>
+      <c r="T8" s="71"/>
+      <c r="U8" s="69"/>
+      <c r="V8" s="69"/>
+      <c r="W8" s="71"/>
+      <c r="X8" s="73"/>
+      <c r="Y8" s="75"/>
       <c r="Z8" s="26"/>
       <c r="AA8" s="26"/>
       <c r="AB8" s="26"/>
     </row>
     <row r="9" spans="1:28" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="74"/>
-      <c r="B9" s="81"/>
-      <c r="C9" s="83"/>
-      <c r="D9" s="83"/>
-      <c r="E9" s="85"/>
-      <c r="F9" s="65" t="s">
+      <c r="A9" s="61"/>
+      <c r="B9" s="63"/>
+      <c r="C9" s="65"/>
+      <c r="D9" s="65"/>
+      <c r="E9" s="67"/>
+      <c r="F9" s="80" t="s">
         <v>34</v>
       </c>
-      <c r="G9" s="65" t="s">
+      <c r="G9" s="80" t="s">
         <v>35</v>
       </c>
-      <c r="H9" s="73" t="s">
+      <c r="H9" s="60" t="s">
         <v>36</v>
       </c>
-      <c r="I9" s="75" t="s">
+      <c r="I9" s="88" t="s">
         <v>37</v>
       </c>
-      <c r="J9" s="66"/>
-      <c r="K9" s="73" t="s">
+      <c r="J9" s="81"/>
+      <c r="K9" s="60" t="s">
         <v>38</v>
       </c>
-      <c r="L9" s="77" t="s">
+      <c r="L9" s="57" t="s">
         <v>39</v>
       </c>
-      <c r="M9" s="78"/>
-      <c r="N9" s="78"/>
-      <c r="O9" s="79"/>
+      <c r="M9" s="59"/>
+      <c r="N9" s="59"/>
+      <c r="O9" s="58"/>
       <c r="P9" s="27"/>
-      <c r="Q9" s="54"/>
-      <c r="R9" s="54"/>
-      <c r="S9" s="54"/>
-      <c r="T9" s="54"/>
-      <c r="U9" s="56"/>
-      <c r="V9" s="56"/>
-      <c r="W9" s="54"/>
-      <c r="X9" s="58"/>
-      <c r="Y9" s="60"/>
+      <c r="Q9" s="71"/>
+      <c r="R9" s="71"/>
+      <c r="S9" s="71"/>
+      <c r="T9" s="71"/>
+      <c r="U9" s="69"/>
+      <c r="V9" s="69"/>
+      <c r="W9" s="71"/>
+      <c r="X9" s="73"/>
+      <c r="Y9" s="75"/>
       <c r="Z9" s="26"/>
       <c r="AA9" s="26"/>
       <c r="AB9" s="26"/>
     </row>
     <row r="10" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="74"/>
-      <c r="B10" s="81"/>
-      <c r="C10" s="83"/>
-      <c r="D10" s="83"/>
-      <c r="E10" s="85"/>
-      <c r="F10" s="66"/>
-      <c r="G10" s="66"/>
-      <c r="H10" s="74"/>
-      <c r="I10" s="76"/>
-      <c r="J10" s="66"/>
-      <c r="K10" s="74"/>
+      <c r="A10" s="61"/>
+      <c r="B10" s="63"/>
+      <c r="C10" s="65"/>
+      <c r="D10" s="65"/>
+      <c r="E10" s="67"/>
+      <c r="F10" s="81"/>
+      <c r="G10" s="81"/>
+      <c r="H10" s="61"/>
+      <c r="I10" s="89"/>
+      <c r="J10" s="81"/>
+      <c r="K10" s="61"/>
       <c r="L10" s="28" t="s">
         <v>40</v>
       </c>
@@ -2525,15 +2541,15 @@
         <v>43</v>
       </c>
       <c r="P10" s="27"/>
-      <c r="Q10" s="54"/>
-      <c r="R10" s="54"/>
-      <c r="S10" s="54"/>
-      <c r="T10" s="54"/>
-      <c r="U10" s="56"/>
-      <c r="V10" s="56"/>
-      <c r="W10" s="54"/>
-      <c r="X10" s="58"/>
-      <c r="Y10" s="60"/>
+      <c r="Q10" s="71"/>
+      <c r="R10" s="71"/>
+      <c r="S10" s="71"/>
+      <c r="T10" s="71"/>
+      <c r="U10" s="69"/>
+      <c r="V10" s="69"/>
+      <c r="W10" s="71"/>
+      <c r="X10" s="73"/>
+      <c r="Y10" s="75"/>
       <c r="Z10" s="26"/>
       <c r="AA10" s="26"/>
       <c r="AB10" s="26"/>
@@ -2678,7 +2694,7 @@
       <c r="Q15" s="33"/>
       <c r="R15" s="33"/>
       <c r="S15" s="33"/>
-      <c r="T15" s="49"/>
+      <c r="T15" s="48"/>
       <c r="U15" s="33"/>
       <c r="V15" s="33"/>
       <c r="W15" s="33"/>
@@ -2688,358 +2704,366 @@
       <c r="AA15" s="26"/>
       <c r="AB15" s="26"/>
     </row>
-    <row r="16" spans="1:28" ht="26.25" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A16" s="26"/>
-      <c r="B16" s="26"/>
-      <c r="C16" s="26"/>
-      <c r="D16" s="26"/>
-      <c r="E16" s="26"/>
-      <c r="F16" s="26"/>
-      <c r="G16" s="26"/>
-      <c r="H16" s="26"/>
-      <c r="I16" s="26"/>
-      <c r="J16" s="26"/>
-      <c r="K16" s="26"/>
-      <c r="L16" s="26"/>
-      <c r="M16" s="26"/>
-      <c r="N16" s="26"/>
-      <c r="O16" s="26"/>
-      <c r="P16" s="26"/>
-      <c r="Q16" s="34"/>
-      <c r="R16" s="34"/>
-      <c r="S16" s="34"/>
-      <c r="T16" s="34"/>
-      <c r="U16" s="34"/>
-      <c r="V16" s="34"/>
-      <c r="W16" s="34"/>
-      <c r="X16" s="34"/>
-      <c r="Y16" s="34"/>
+    <row r="16" spans="1:28" ht="48" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="93"/>
+      <c r="B16" s="93"/>
+      <c r="C16" s="93"/>
+      <c r="D16" s="93"/>
+      <c r="E16" s="93"/>
+      <c r="F16" s="93"/>
+      <c r="G16" s="93"/>
+      <c r="H16" s="94"/>
+      <c r="I16" s="93"/>
+      <c r="J16" s="94"/>
+      <c r="K16" s="95"/>
+      <c r="L16" s="96"/>
+      <c r="M16" s="93"/>
+      <c r="N16" s="93"/>
+      <c r="O16" s="93"/>
+      <c r="P16" s="93"/>
+      <c r="Q16" s="97"/>
+      <c r="R16" s="97"/>
+      <c r="S16" s="97"/>
+      <c r="T16" s="97"/>
+      <c r="U16" s="97"/>
+      <c r="V16" s="97"/>
+      <c r="W16" s="97"/>
+      <c r="X16" s="97"/>
+      <c r="Y16" s="97"/>
       <c r="Z16" s="26"/>
       <c r="AA16" s="26"/>
       <c r="AB16" s="26"/>
     </row>
-    <row r="17" spans="1:28" ht="26.25" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A17" s="35"/>
-      <c r="B17" s="26"/>
-      <c r="C17" s="26"/>
-      <c r="D17" s="26"/>
-      <c r="E17" s="26"/>
-      <c r="F17" s="26"/>
-      <c r="G17" s="26"/>
-      <c r="H17" s="26"/>
-      <c r="I17" s="26"/>
-      <c r="J17" s="26"/>
-      <c r="K17" s="36"/>
-      <c r="L17" s="36"/>
-      <c r="M17" s="36"/>
-      <c r="N17" s="36"/>
-      <c r="O17" s="50" t="s">
-        <v>44</v>
-      </c>
-      <c r="P17" s="51"/>
-      <c r="Q17" s="37"/>
-      <c r="R17" s="37"/>
-      <c r="S17" s="37"/>
-      <c r="T17" s="37"/>
-      <c r="U17" s="37"/>
-      <c r="V17" s="37"/>
-      <c r="W17" s="37"/>
-      <c r="X17" s="37"/>
-      <c r="Y17" s="37"/>
+    <row r="17" spans="1:28" ht="48" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="93"/>
+      <c r="B17" s="93"/>
+      <c r="C17" s="93"/>
+      <c r="D17" s="93"/>
+      <c r="E17" s="93"/>
+      <c r="F17" s="93"/>
+      <c r="G17" s="93"/>
+      <c r="H17" s="94"/>
+      <c r="I17" s="93"/>
+      <c r="J17" s="94"/>
+      <c r="K17" s="95"/>
+      <c r="L17" s="96"/>
+      <c r="M17" s="93"/>
+      <c r="N17" s="93"/>
+      <c r="O17" s="93"/>
+      <c r="P17" s="93"/>
+      <c r="Q17" s="97"/>
+      <c r="R17" s="97"/>
+      <c r="S17" s="97"/>
+      <c r="T17" s="97"/>
+      <c r="U17" s="97"/>
+      <c r="V17" s="97"/>
+      <c r="W17" s="97"/>
+      <c r="X17" s="97"/>
+      <c r="Y17" s="97"/>
       <c r="Z17" s="26"/>
       <c r="AA17" s="26"/>
       <c r="AB17" s="26"/>
     </row>
-    <row r="18" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A18" s="26"/>
-      <c r="B18" s="26"/>
-      <c r="C18" s="26"/>
-      <c r="D18" s="26"/>
-      <c r="E18" s="26"/>
-      <c r="F18" s="26"/>
-      <c r="G18" s="26"/>
-      <c r="H18" s="26"/>
-      <c r="I18" s="26"/>
-      <c r="J18" s="26"/>
-      <c r="K18" s="26"/>
-      <c r="L18" s="26"/>
-      <c r="M18" s="26"/>
-      <c r="N18" s="26"/>
-      <c r="O18" s="26"/>
-      <c r="P18" s="26"/>
-      <c r="Q18" s="26"/>
-      <c r="R18" s="26"/>
-      <c r="S18" s="26"/>
-      <c r="T18" s="26"/>
-      <c r="U18" s="26"/>
-      <c r="V18" s="26"/>
-      <c r="W18" s="26"/>
-      <c r="X18" s="26"/>
-      <c r="Y18" s="26"/>
+    <row r="18" spans="1:28" ht="48" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="93"/>
+      <c r="B18" s="93"/>
+      <c r="C18" s="93"/>
+      <c r="D18" s="93"/>
+      <c r="E18" s="93"/>
+      <c r="F18" s="93"/>
+      <c r="G18" s="93"/>
+      <c r="H18" s="30"/>
+      <c r="I18" s="29"/>
+      <c r="J18" s="30"/>
+      <c r="K18" s="31"/>
+      <c r="L18" s="29"/>
+      <c r="M18" s="29"/>
+      <c r="N18" s="29"/>
+      <c r="O18" s="29"/>
+      <c r="P18" s="29"/>
+      <c r="Q18" s="33"/>
+      <c r="R18" s="33"/>
+      <c r="S18" s="33"/>
+      <c r="T18" s="33"/>
+      <c r="U18" s="33"/>
+      <c r="V18" s="33"/>
+      <c r="W18" s="33"/>
+      <c r="X18" s="33"/>
+      <c r="Y18" s="33"/>
       <c r="Z18" s="26"/>
       <c r="AA18" s="26"/>
       <c r="AB18" s="26"/>
     </row>
-    <row r="19" spans="1:28" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A19" s="38" t="s">
-        <v>45</v>
-      </c>
-      <c r="B19" s="39"/>
-      <c r="C19" s="40"/>
-      <c r="D19" s="26"/>
-      <c r="E19" s="26"/>
-      <c r="F19" s="26"/>
-      <c r="G19" s="26"/>
-      <c r="H19" s="26"/>
-      <c r="I19" s="26"/>
-      <c r="J19" s="26"/>
-      <c r="K19" s="26"/>
-      <c r="L19" s="26"/>
-      <c r="M19" s="26"/>
-      <c r="N19" s="26"/>
-      <c r="O19" s="26"/>
-      <c r="P19" s="26"/>
-      <c r="Q19" s="26"/>
-      <c r="R19" s="26"/>
-      <c r="S19" s="41"/>
-      <c r="T19" s="42"/>
-      <c r="U19" s="42"/>
-      <c r="V19" s="42"/>
-      <c r="W19" s="42"/>
-      <c r="X19" s="42"/>
-      <c r="Y19" s="43"/>
+    <row r="19" spans="1:28" ht="48" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="93"/>
+      <c r="B19" s="93"/>
+      <c r="C19" s="93"/>
+      <c r="D19" s="93"/>
+      <c r="E19" s="93"/>
+      <c r="F19" s="93"/>
+      <c r="G19" s="93"/>
+      <c r="H19" s="30"/>
+      <c r="I19" s="29"/>
+      <c r="J19" s="30"/>
+      <c r="K19" s="31"/>
+      <c r="L19" s="32"/>
+      <c r="M19" s="29"/>
+      <c r="N19" s="29"/>
+      <c r="O19" s="29"/>
+      <c r="P19" s="29"/>
+      <c r="Q19" s="33"/>
+      <c r="R19" s="33"/>
+      <c r="S19" s="33"/>
+      <c r="T19" s="33"/>
+      <c r="U19" s="33"/>
+      <c r="V19" s="33"/>
+      <c r="W19" s="33"/>
+      <c r="X19" s="33"/>
+      <c r="Y19" s="33"/>
       <c r="Z19" s="26"/>
       <c r="AA19" s="26"/>
       <c r="AB19" s="26"/>
     </row>
-    <row r="20" spans="1:28" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A20" s="39"/>
-      <c r="B20" s="39"/>
-      <c r="C20" s="40"/>
-      <c r="D20" s="26"/>
-      <c r="E20" s="26"/>
-      <c r="F20" s="26"/>
-      <c r="G20" s="26"/>
-      <c r="H20" s="26"/>
-      <c r="I20" s="26"/>
-      <c r="J20" s="26"/>
-      <c r="K20" s="26"/>
-      <c r="L20" s="26"/>
-      <c r="M20" s="26"/>
-      <c r="N20" s="26"/>
-      <c r="O20" s="26"/>
-      <c r="P20" s="26"/>
-      <c r="Q20" s="35"/>
-      <c r="R20" s="35"/>
-      <c r="S20" s="41"/>
-      <c r="T20" s="42"/>
-      <c r="U20" s="42"/>
-      <c r="V20" s="42"/>
-      <c r="W20" s="42"/>
-      <c r="X20" s="42"/>
-      <c r="Y20" s="43"/>
+    <row r="20" spans="1:28" ht="48" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="93"/>
+      <c r="B20" s="93"/>
+      <c r="C20" s="93"/>
+      <c r="D20" s="93"/>
+      <c r="E20" s="93"/>
+      <c r="F20" s="93"/>
+      <c r="G20" s="93"/>
+      <c r="H20" s="30"/>
+      <c r="I20" s="29"/>
+      <c r="J20" s="30"/>
+      <c r="K20" s="31"/>
+      <c r="L20" s="32"/>
+      <c r="M20" s="29"/>
+      <c r="N20" s="29"/>
+      <c r="O20" s="29"/>
+      <c r="P20" s="29"/>
+      <c r="Q20" s="33"/>
+      <c r="R20" s="33"/>
+      <c r="S20" s="33"/>
+      <c r="T20" s="48"/>
+      <c r="U20" s="33"/>
+      <c r="V20" s="33"/>
+      <c r="W20" s="33"/>
+      <c r="X20" s="33"/>
+      <c r="Y20" s="33"/>
       <c r="Z20" s="26"/>
       <c r="AA20" s="26"/>
       <c r="AB20" s="26"/>
     </row>
-    <row r="21" spans="1:28" ht="20.25" x14ac:dyDescent="0.3">
-      <c r="A21" s="44" t="s">
-        <v>46</v>
-      </c>
-      <c r="B21" s="39"/>
-      <c r="C21" s="40"/>
-      <c r="D21" s="26"/>
-      <c r="E21" s="26"/>
-      <c r="F21" s="26"/>
-      <c r="G21" s="52" t="s">
-        <v>47</v>
-      </c>
-      <c r="H21" s="52"/>
-      <c r="I21" s="26"/>
-      <c r="J21" s="26"/>
-      <c r="K21" s="26"/>
-      <c r="L21" s="45"/>
-      <c r="M21" s="52" t="s">
-        <v>48</v>
-      </c>
-      <c r="N21" s="52"/>
-      <c r="O21" s="26"/>
-      <c r="P21" s="26"/>
-      <c r="Q21" s="26"/>
-      <c r="R21" s="26"/>
-      <c r="S21" s="41"/>
-      <c r="T21" s="42"/>
-      <c r="U21" s="42"/>
-      <c r="V21" s="42"/>
-      <c r="W21" s="42"/>
-      <c r="X21" s="42"/>
-      <c r="Y21" s="43"/>
+    <row r="21" spans="1:28" ht="48" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="93"/>
+      <c r="B21" s="93"/>
+      <c r="C21" s="93"/>
+      <c r="D21" s="93"/>
+      <c r="E21" s="93"/>
+      <c r="F21" s="93"/>
+      <c r="G21" s="93"/>
+      <c r="H21" s="30"/>
+      <c r="I21" s="29"/>
+      <c r="J21" s="30"/>
+      <c r="K21" s="31"/>
+      <c r="L21" s="32"/>
+      <c r="M21" s="29"/>
+      <c r="N21" s="29"/>
+      <c r="O21" s="29"/>
+      <c r="P21" s="29"/>
+      <c r="Q21" s="33"/>
+      <c r="R21" s="33"/>
+      <c r="S21" s="33"/>
+      <c r="T21" s="33"/>
+      <c r="U21" s="33"/>
+      <c r="V21" s="33"/>
+      <c r="W21" s="33"/>
+      <c r="X21" s="33"/>
+      <c r="Y21" s="33"/>
       <c r="Z21" s="26"/>
       <c r="AA21" s="26"/>
       <c r="AB21" s="26"/>
     </row>
-    <row r="22" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A22" s="39"/>
-      <c r="B22" s="39"/>
-      <c r="C22" s="40"/>
-      <c r="D22" s="26"/>
-      <c r="O22" s="26"/>
-      <c r="P22" s="26"/>
-      <c r="S22" s="26"/>
-      <c r="T22" s="26"/>
-      <c r="U22" s="26"/>
-      <c r="V22" s="26"/>
-      <c r="W22" s="26"/>
-      <c r="X22" s="26"/>
-      <c r="Y22" s="26"/>
+    <row r="22" spans="1:28" ht="48" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="93"/>
+      <c r="B22" s="93"/>
+      <c r="C22" s="93"/>
+      <c r="D22" s="93"/>
+      <c r="E22" s="93"/>
+      <c r="F22" s="93"/>
+      <c r="G22" s="93"/>
+      <c r="H22" s="30"/>
+      <c r="I22" s="29"/>
+      <c r="J22" s="30"/>
+      <c r="K22" s="31"/>
+      <c r="L22" s="32"/>
+      <c r="M22" s="29"/>
+      <c r="N22" s="29"/>
+      <c r="O22" s="29"/>
+      <c r="P22" s="29"/>
+      <c r="Q22" s="33"/>
+      <c r="R22" s="33"/>
+      <c r="S22" s="33"/>
+      <c r="T22" s="33"/>
+      <c r="U22" s="33"/>
+      <c r="V22" s="33"/>
+      <c r="W22" s="33"/>
+      <c r="X22" s="33"/>
+      <c r="Y22" s="33"/>
       <c r="Z22" s="26"/>
       <c r="AA22" s="26"/>
       <c r="AB22" s="26"/>
     </row>
-    <row r="23" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A23" s="44" t="str">
-        <f>+'[1]ANEXO NP1'!A78</f>
-        <v>MES: FEBRERO   AÑO: 2025</v>
-      </c>
-      <c r="B23" s="39"/>
-      <c r="C23" s="40"/>
-      <c r="D23" s="26"/>
-      <c r="E23" s="26"/>
-      <c r="F23" s="26"/>
-      <c r="G23" s="26"/>
-      <c r="H23" s="26"/>
-      <c r="I23" s="26"/>
-      <c r="J23" s="26"/>
-      <c r="K23" s="46"/>
-      <c r="L23" s="26"/>
-      <c r="M23" s="46"/>
-      <c r="N23" s="1"/>
-      <c r="O23" s="46"/>
-      <c r="P23" s="26"/>
-      <c r="S23" s="26"/>
-      <c r="T23" s="1"/>
-      <c r="U23" s="1"/>
-      <c r="V23" s="1"/>
-      <c r="W23" s="1"/>
-      <c r="X23" s="1"/>
-      <c r="Y23" s="26"/>
+    <row r="23" spans="1:28" ht="48" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="93"/>
+      <c r="B23" s="93"/>
+      <c r="C23" s="93"/>
+      <c r="D23" s="93"/>
+      <c r="E23" s="93"/>
+      <c r="F23" s="93"/>
+      <c r="G23" s="93"/>
+      <c r="H23" s="30"/>
+      <c r="I23" s="29"/>
+      <c r="J23" s="30"/>
+      <c r="K23" s="31"/>
+      <c r="L23" s="29"/>
+      <c r="M23" s="29"/>
+      <c r="N23" s="29"/>
+      <c r="O23" s="29"/>
+      <c r="P23" s="29"/>
+      <c r="Q23" s="33"/>
+      <c r="R23" s="33"/>
+      <c r="S23" s="33"/>
+      <c r="T23" s="33"/>
+      <c r="U23" s="33"/>
+      <c r="V23" s="33"/>
+      <c r="W23" s="33"/>
+      <c r="X23" s="33"/>
+      <c r="Y23" s="33"/>
       <c r="Z23" s="26"/>
       <c r="AA23" s="26"/>
       <c r="AB23" s="26"/>
     </row>
-    <row r="24" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A24" s="1"/>
-      <c r="B24" s="26"/>
-      <c r="K24" s="26"/>
-      <c r="L24" s="26"/>
-      <c r="M24" s="26"/>
-      <c r="N24" s="26"/>
-      <c r="O24" s="26"/>
-      <c r="P24" s="26"/>
-      <c r="S24" s="26"/>
-      <c r="T24" s="26"/>
-      <c r="U24" s="26"/>
-      <c r="V24" s="26"/>
-      <c r="W24" s="26"/>
-      <c r="X24" s="26"/>
-      <c r="Y24" s="26"/>
+    <row r="24" spans="1:28" ht="48" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="93"/>
+      <c r="B24" s="93"/>
+      <c r="C24" s="93"/>
+      <c r="D24" s="93"/>
+      <c r="E24" s="93"/>
+      <c r="F24" s="93"/>
+      <c r="G24" s="93"/>
+      <c r="H24" s="30"/>
+      <c r="I24" s="29"/>
+      <c r="J24" s="30"/>
+      <c r="K24" s="31"/>
+      <c r="L24" s="32"/>
+      <c r="M24" s="29"/>
+      <c r="N24" s="29"/>
+      <c r="O24" s="29"/>
+      <c r="P24" s="29"/>
+      <c r="Q24" s="33"/>
+      <c r="R24" s="33"/>
+      <c r="S24" s="33"/>
+      <c r="T24" s="33"/>
+      <c r="U24" s="33"/>
+      <c r="V24" s="33"/>
+      <c r="W24" s="33"/>
+      <c r="X24" s="33"/>
+      <c r="Y24" s="33"/>
       <c r="Z24" s="26"/>
       <c r="AA24" s="26"/>
       <c r="AB24" s="26"/>
     </row>
-    <row r="25" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A25" s="1"/>
-      <c r="B25" s="26"/>
-      <c r="C25" s="26"/>
-      <c r="D25" s="26"/>
-      <c r="E25" s="26"/>
-      <c r="F25" s="26"/>
-      <c r="G25" s="26"/>
-      <c r="H25" s="26"/>
-      <c r="I25" s="26"/>
-      <c r="J25" s="26"/>
-      <c r="K25" s="26"/>
-      <c r="L25" s="26"/>
-      <c r="M25" s="26"/>
-      <c r="N25" s="26"/>
-      <c r="O25" s="26"/>
-      <c r="P25" s="26"/>
-      <c r="Q25" s="26"/>
-      <c r="R25" s="26"/>
-      <c r="S25" s="26"/>
-      <c r="T25" s="26"/>
-      <c r="U25" s="26"/>
-      <c r="V25" s="26"/>
-      <c r="W25" s="26"/>
-      <c r="X25" s="26"/>
-      <c r="Y25" s="47" t="s">
-        <v>49</v>
-      </c>
+    <row r="25" spans="1:28" ht="48" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="93"/>
+      <c r="B25" s="93"/>
+      <c r="C25" s="93"/>
+      <c r="D25" s="93"/>
+      <c r="E25" s="93"/>
+      <c r="F25" s="93"/>
+      <c r="G25" s="93"/>
+      <c r="H25" s="30"/>
+      <c r="I25" s="29"/>
+      <c r="J25" s="30"/>
+      <c r="K25" s="31"/>
+      <c r="L25" s="32"/>
+      <c r="M25" s="29"/>
+      <c r="N25" s="29"/>
+      <c r="O25" s="29"/>
+      <c r="P25" s="29"/>
+      <c r="Q25" s="33"/>
+      <c r="R25" s="33"/>
+      <c r="T25" s="48"/>
+      <c r="U25" s="33"/>
+      <c r="V25" s="33"/>
+      <c r="W25" s="33"/>
+      <c r="X25" s="33"/>
+      <c r="Y25" s="33"/>
       <c r="Z25" s="26"/>
       <c r="AA25" s="26"/>
       <c r="AB25" s="26"/>
     </row>
-    <row r="26" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A26" s="35"/>
-      <c r="B26" s="26"/>
-      <c r="C26" s="26"/>
-      <c r="D26" s="26"/>
-      <c r="E26" s="26"/>
-      <c r="F26" s="26"/>
-      <c r="G26" s="26"/>
-      <c r="H26" s="26"/>
-      <c r="I26" s="26"/>
-      <c r="J26" s="26"/>
-      <c r="K26" s="26"/>
-      <c r="L26" s="26"/>
-      <c r="M26" s="26"/>
-      <c r="N26" s="26"/>
-      <c r="O26" s="26"/>
-      <c r="P26" s="26"/>
-      <c r="Q26" s="26"/>
-      <c r="R26" s="26"/>
-      <c r="S26" s="26"/>
-      <c r="T26" s="26"/>
-      <c r="U26" s="26"/>
-      <c r="V26" s="26"/>
-      <c r="W26" s="26"/>
-      <c r="X26" s="26"/>
-      <c r="Y26" s="26"/>
+    <row r="26" spans="1:28" ht="48" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="93"/>
+      <c r="B26" s="93"/>
+      <c r="C26" s="93"/>
+      <c r="D26" s="93"/>
+      <c r="E26" s="93"/>
+      <c r="F26" s="93"/>
+      <c r="G26" s="93"/>
+      <c r="H26" s="30"/>
+      <c r="I26" s="29"/>
+      <c r="J26" s="30"/>
+      <c r="K26" s="31"/>
+      <c r="L26" s="32"/>
+      <c r="M26" s="29"/>
+      <c r="N26" s="29"/>
+      <c r="O26" s="29"/>
+      <c r="P26" s="29"/>
+      <c r="Q26" s="33"/>
+      <c r="R26" s="33"/>
+      <c r="S26" s="33"/>
+      <c r="T26" s="48"/>
+      <c r="U26" s="33"/>
+      <c r="V26" s="33"/>
+      <c r="W26" s="33"/>
+      <c r="X26" s="33"/>
+      <c r="Y26" s="33"/>
       <c r="Z26" s="26"/>
       <c r="AA26" s="26"/>
       <c r="AB26" s="26"/>
     </row>
-    <row r="27" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A27" s="26"/>
-      <c r="B27" s="26"/>
-      <c r="C27" s="26"/>
-      <c r="D27" s="26"/>
-      <c r="E27" s="26"/>
-      <c r="F27" s="26"/>
-      <c r="G27" s="26"/>
-      <c r="H27" s="26"/>
-      <c r="I27" s="26"/>
-      <c r="J27" s="26"/>
-      <c r="K27" s="26"/>
-      <c r="L27" s="26"/>
-      <c r="M27" s="26"/>
-      <c r="N27" s="26"/>
-      <c r="O27" s="26"/>
-      <c r="P27" s="26"/>
-      <c r="Q27" s="26"/>
-      <c r="R27" s="26"/>
-      <c r="S27" s="35"/>
-      <c r="T27" s="26"/>
-      <c r="U27" s="26"/>
-      <c r="V27" s="26"/>
-      <c r="W27" s="26"/>
-      <c r="X27" s="26"/>
-      <c r="Y27" s="26"/>
+    <row r="27" spans="1:28" ht="48" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="93"/>
+      <c r="B27" s="93"/>
+      <c r="C27" s="93"/>
+      <c r="D27" s="93"/>
+      <c r="E27" s="93"/>
+      <c r="F27" s="93"/>
+      <c r="G27" s="93"/>
+      <c r="H27" s="30"/>
+      <c r="I27" s="29"/>
+      <c r="J27" s="30"/>
+      <c r="K27" s="31"/>
+      <c r="L27" s="32"/>
+      <c r="M27" s="29"/>
+      <c r="N27" s="29"/>
+      <c r="O27" s="29"/>
+      <c r="P27" s="29"/>
+      <c r="Q27" s="33"/>
+      <c r="R27" s="33"/>
+      <c r="S27" s="33"/>
+      <c r="T27" s="48"/>
+      <c r="U27" s="33"/>
+      <c r="V27" s="33"/>
+      <c r="W27" s="33"/>
+      <c r="X27" s="33"/>
+      <c r="Y27" s="33"/>
       <c r="Z27" s="26"/>
       <c r="AA27" s="26"/>
       <c r="AB27" s="26"/>
     </row>
-    <row r="28" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="26"/>
       <c r="B28" s="26"/>
       <c r="C28" s="26"/>
@@ -3069,7 +3093,7 @@
       <c r="AA28" s="26"/>
       <c r="AB28" s="26"/>
     </row>
-    <row r="29" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:28" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="26"/>
       <c r="B29" s="26"/>
       <c r="C29" s="26"/>
@@ -3096,22 +3120,253 @@
       <c r="X29" s="26"/>
       <c r="Y29" s="26"/>
       <c r="Z29" s="26"/>
-      <c r="AA29" s="48"/>
+      <c r="AA29" s="47"/>
       <c r="AB29" s="26"/>
     </row>
+    <row r="30" spans="1:28" ht="26.25" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A30" s="34"/>
+      <c r="B30" s="26"/>
+      <c r="C30" s="26"/>
+      <c r="D30" s="26"/>
+      <c r="E30" s="26"/>
+      <c r="F30" s="26"/>
+      <c r="G30" s="26"/>
+      <c r="H30" s="26"/>
+      <c r="I30" s="26"/>
+      <c r="J30" s="26"/>
+      <c r="K30" s="35"/>
+      <c r="L30" s="35"/>
+      <c r="M30" s="35"/>
+      <c r="N30" s="35"/>
+      <c r="O30" s="49" t="s">
+        <v>44</v>
+      </c>
+      <c r="P30" s="50"/>
+      <c r="Q30" s="36"/>
+      <c r="R30" s="36"/>
+      <c r="S30" s="36"/>
+      <c r="T30" s="36"/>
+      <c r="U30" s="36"/>
+      <c r="V30" s="36"/>
+      <c r="W30" s="36"/>
+      <c r="X30" s="36"/>
+      <c r="Y30" s="36"/>
+    </row>
+    <row r="31" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A31" s="26"/>
+      <c r="B31" s="26"/>
+      <c r="C31" s="26"/>
+      <c r="D31" s="26"/>
+      <c r="E31" s="26"/>
+      <c r="F31" s="26"/>
+      <c r="G31" s="26"/>
+      <c r="H31" s="26"/>
+      <c r="I31" s="26"/>
+      <c r="J31" s="26"/>
+      <c r="K31" s="26"/>
+      <c r="L31" s="26"/>
+      <c r="M31" s="26"/>
+      <c r="N31" s="26"/>
+      <c r="O31" s="26"/>
+      <c r="P31" s="26"/>
+      <c r="Q31" s="26"/>
+      <c r="R31" s="26"/>
+      <c r="S31" s="26"/>
+      <c r="T31" s="26"/>
+      <c r="U31" s="26"/>
+      <c r="V31" s="26"/>
+      <c r="W31" s="26"/>
+      <c r="X31" s="26"/>
+      <c r="Y31" s="26"/>
+    </row>
+    <row r="32" spans="1:28" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A32" s="37" t="s">
+        <v>45</v>
+      </c>
+      <c r="B32" s="38"/>
+      <c r="C32" s="39"/>
+      <c r="D32" s="26"/>
+      <c r="E32" s="26"/>
+      <c r="F32" s="26"/>
+      <c r="G32" s="26"/>
+      <c r="H32" s="26"/>
+      <c r="I32" s="26"/>
+      <c r="J32" s="26"/>
+      <c r="K32" s="26"/>
+      <c r="L32" s="26"/>
+      <c r="M32" s="26"/>
+      <c r="N32" s="26"/>
+      <c r="O32" s="26"/>
+      <c r="P32" s="26"/>
+      <c r="Q32" s="26"/>
+      <c r="R32" s="26"/>
+      <c r="S32" s="40"/>
+      <c r="T32" s="41"/>
+      <c r="U32" s="41"/>
+      <c r="V32" s="41"/>
+      <c r="W32" s="41"/>
+      <c r="X32" s="41"/>
+      <c r="Y32" s="42"/>
+    </row>
+    <row r="33" spans="1:25" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A33" s="38"/>
+      <c r="B33" s="38"/>
+      <c r="C33" s="39"/>
+      <c r="D33" s="26"/>
+      <c r="E33" s="26"/>
+      <c r="F33" s="26"/>
+      <c r="G33" s="26"/>
+      <c r="H33" s="26"/>
+      <c r="I33" s="26"/>
+      <c r="J33" s="26"/>
+      <c r="K33" s="26"/>
+      <c r="L33" s="26"/>
+      <c r="M33" s="26"/>
+      <c r="N33" s="26"/>
+      <c r="O33" s="26"/>
+      <c r="P33" s="26"/>
+      <c r="Q33" s="34"/>
+      <c r="R33" s="34"/>
+      <c r="S33" s="40"/>
+      <c r="T33" s="41"/>
+      <c r="U33" s="41"/>
+      <c r="V33" s="41"/>
+      <c r="W33" s="41"/>
+      <c r="X33" s="41"/>
+      <c r="Y33" s="42"/>
+    </row>
+    <row r="34" spans="1:25" ht="20.25" x14ac:dyDescent="0.3">
+      <c r="A34" s="43" t="s">
+        <v>46</v>
+      </c>
+      <c r="B34" s="38"/>
+      <c r="C34" s="39"/>
+      <c r="D34" s="26"/>
+      <c r="E34" s="26"/>
+      <c r="F34" s="26"/>
+      <c r="G34" s="90" t="s">
+        <v>47</v>
+      </c>
+      <c r="H34" s="90"/>
+      <c r="I34" s="26"/>
+      <c r="J34" s="26"/>
+      <c r="K34" s="26"/>
+      <c r="L34" s="44"/>
+      <c r="M34" s="90" t="s">
+        <v>48</v>
+      </c>
+      <c r="N34" s="90"/>
+      <c r="O34" s="26"/>
+      <c r="P34" s="26"/>
+      <c r="Q34" s="26"/>
+      <c r="R34" s="26"/>
+      <c r="S34" s="40"/>
+      <c r="T34" s="41"/>
+      <c r="U34" s="41"/>
+      <c r="V34" s="41"/>
+      <c r="W34" s="41"/>
+      <c r="X34" s="41"/>
+      <c r="Y34" s="42"/>
+    </row>
+    <row r="35" spans="1:25" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="38"/>
+      <c r="B35" s="38"/>
+      <c r="C35" s="39"/>
+      <c r="D35" s="26"/>
+      <c r="O35" s="26"/>
+      <c r="P35" s="26"/>
+      <c r="S35" s="26"/>
+      <c r="T35" s="26"/>
+      <c r="U35" s="26"/>
+      <c r="V35" s="26"/>
+      <c r="W35" s="26"/>
+      <c r="X35" s="26"/>
+      <c r="Y35" s="26"/>
+    </row>
+    <row r="36" spans="1:25" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="43" t="str">
+        <f>+'[1]ANEXO NP1'!A78</f>
+        <v>MES: FEBRERO   AÑO: 2025</v>
+      </c>
+      <c r="B36" s="38"/>
+      <c r="C36" s="39"/>
+      <c r="D36" s="26"/>
+      <c r="E36" s="26"/>
+      <c r="F36" s="26"/>
+      <c r="G36" s="26"/>
+      <c r="H36" s="26"/>
+      <c r="I36" s="26"/>
+      <c r="J36" s="26"/>
+      <c r="K36" s="45"/>
+      <c r="L36" s="26"/>
+      <c r="M36" s="45"/>
+      <c r="N36" s="1"/>
+      <c r="O36" s="45"/>
+      <c r="P36" s="26"/>
+      <c r="S36" s="26"/>
+      <c r="T36" s="1"/>
+      <c r="U36" s="1"/>
+      <c r="V36" s="1"/>
+      <c r="W36" s="1"/>
+      <c r="X36" s="1"/>
+      <c r="Y36" s="26"/>
+    </row>
+    <row r="37" spans="1:25" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="1"/>
+      <c r="B37" s="26"/>
+      <c r="K37" s="26"/>
+      <c r="L37" s="26"/>
+      <c r="M37" s="26"/>
+      <c r="N37" s="26"/>
+      <c r="O37" s="26"/>
+      <c r="P37" s="26"/>
+      <c r="S37" s="26"/>
+      <c r="T37" s="26"/>
+      <c r="U37" s="26"/>
+      <c r="V37" s="26"/>
+      <c r="W37" s="26"/>
+      <c r="X37" s="26"/>
+      <c r="Y37" s="26"/>
+    </row>
+    <row r="38" spans="1:25" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="1"/>
+      <c r="B38" s="26"/>
+      <c r="C38" s="26"/>
+      <c r="D38" s="26"/>
+      <c r="E38" s="26"/>
+      <c r="F38" s="26"/>
+      <c r="G38" s="26"/>
+      <c r="H38" s="26"/>
+      <c r="I38" s="26"/>
+      <c r="J38" s="26"/>
+      <c r="K38" s="26"/>
+      <c r="L38" s="26"/>
+      <c r="M38" s="26"/>
+      <c r="N38" s="26"/>
+      <c r="O38" s="26"/>
+      <c r="P38" s="26"/>
+      <c r="Q38" s="26"/>
+      <c r="R38" s="26"/>
+      <c r="S38" s="26"/>
+      <c r="T38" s="26"/>
+      <c r="U38" s="26"/>
+      <c r="V38" s="26"/>
+      <c r="W38" s="26"/>
+      <c r="X38" s="26"/>
+      <c r="Y38" s="46" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="39" spans="1:25" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
-  <mergeCells count="33">
-    <mergeCell ref="O2:Y2"/>
-    <mergeCell ref="O3:Y3"/>
-    <mergeCell ref="O4:Y4"/>
-    <mergeCell ref="F6:G6"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="K6:O6"/>
-    <mergeCell ref="A7:A10"/>
-    <mergeCell ref="B7:B10"/>
-    <mergeCell ref="C7:C10"/>
-    <mergeCell ref="D7:D10"/>
-    <mergeCell ref="E7:E10"/>
+  <mergeCells count="32">
+    <mergeCell ref="G34:H34"/>
+    <mergeCell ref="M34:N34"/>
+    <mergeCell ref="T7:T10"/>
+    <mergeCell ref="U7:U10"/>
+    <mergeCell ref="F7:G8"/>
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="G9:G10"/>
     <mergeCell ref="V7:V10"/>
     <mergeCell ref="W7:W10"/>
     <mergeCell ref="X7:X10"/>
@@ -3126,14 +3381,17 @@
     <mergeCell ref="I9:I10"/>
     <mergeCell ref="K9:K10"/>
     <mergeCell ref="L9:O9"/>
-    <mergeCell ref="O17:P17"/>
-    <mergeCell ref="G21:H21"/>
-    <mergeCell ref="M21:N21"/>
-    <mergeCell ref="T7:T10"/>
-    <mergeCell ref="U7:U10"/>
-    <mergeCell ref="F7:G8"/>
-    <mergeCell ref="F9:F10"/>
-    <mergeCell ref="G9:G10"/>
+    <mergeCell ref="A7:A10"/>
+    <mergeCell ref="B7:B10"/>
+    <mergeCell ref="C7:C10"/>
+    <mergeCell ref="D7:D10"/>
+    <mergeCell ref="E7:E10"/>
+    <mergeCell ref="O2:Y2"/>
+    <mergeCell ref="O3:Y3"/>
+    <mergeCell ref="O4:Y4"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="K6:O6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="35" orientation="landscape" r:id="rId1"/>

</xml_diff>

<commit_message>
feat: implementar generación de hoja de anexo para nómina de pago del personal administrativo, mejorando la organización de datos y la presentación de reportes generados
</commit_message>
<xml_diff>
--- a/src/core/excel/templates/ANEXO NOMINA DE PAGO PERSONAL ADMINISTRATIVO.xlsx
+++ b/src/core/excel/templates/ANEXO NOMINA DE PAGO PERSONAL ADMINISTRATIVO.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\david\OneDrive\Documentos\Codigo\san-miguel-porres-backend\src\core\excel\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B46FF5FD-834C-423F-BEE9-AFF08AEC7C41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7292059E-17BA-4D63-A3C7-F726BBC74BD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
   <si>
     <t>ANEXO-NP2-A</t>
   </si>
@@ -196,6 +196,13 @@
   </si>
   <si>
     <t>ANALISIS / JULIO 2023</t>
+  </si>
+  <si>
+    <t>CARGO</t>
+  </si>
+  <si>
+    <t>Nº HORAS
+SEMANAl</t>
   </si>
 </sst>
 </file>
@@ -476,19 +483,6 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
       <top/>
       <bottom/>
       <diagonal/>
@@ -503,6 +497,19 @@
       <top style="thin">
         <color indexed="64"/>
       </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
@@ -514,7 +521,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="101">
+  <cellXfs count="100">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -584,27 +591,21 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="15" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="1" applyBorder="1"/>
-    <xf numFmtId="4" fontId="12" fillId="0" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="1" applyBorder="1"/>
+    <xf numFmtId="4" fontId="12" fillId="0" borderId="15" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1"/>
@@ -641,7 +642,7 @@
     <xf numFmtId="17" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="4" fontId="16" fillId="0" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="4" fontId="16" fillId="0" borderId="15" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
@@ -650,6 +651,9 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="15" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="4" fontId="12" fillId="0" borderId="15" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -659,6 +663,15 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -680,49 +693,49 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -740,7 +753,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -767,6 +780,12 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -776,18 +795,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="4" fontId="12" fillId="0" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="4" fontId="16" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -884,85 +892,6 @@
               <a:cs typeface="Times New Roman"/>
             </a:rPr>
             <a:t>DOCENTE</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>192405</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>635</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>36296</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="3" name="Texto 6">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{ED6608B6-6C74-4BF0-9CFC-589A1CF390CD}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1">
-          <a:spLocks noChangeArrowheads="1"/>
-        </xdr:cNvSpPr>
-      </xdr:nvSpPr>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="13677900" y="2240280"/>
-          <a:ext cx="762635" cy="986891"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="1">
-          <a:noFill/>
-          <a:miter lim="800000"/>
-          <a:headEnd/>
-          <a:tailEnd/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" vert="vert270" wrap="square" lIns="36576" tIns="27432" rIns="36576" bIns="27432" anchor="ctr" upright="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="es-VE" sz="1300" b="1" i="0" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Times New Roman"/>
-              <a:cs typeface="Times New Roman"/>
-            </a:rPr>
-            <a:t>Nº HORAS</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="ctr" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="es-VE" sz="1300" b="1" i="0" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Times New Roman"/>
-              <a:cs typeface="Times New Roman"/>
-            </a:rPr>
-            <a:t>SEMANAl.</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -1091,70 +1020,6 @@
           </a:ext>
         </a:extLst>
       </xdr:spPr>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>41275</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>310398</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>130175</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="6" name="Texto 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{156B315A-E374-4558-9302-AD57B08AB33E}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1">
-          <a:spLocks noChangeArrowheads="1"/>
-        </xdr:cNvSpPr>
-      </xdr:nvSpPr>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="4232275" y="2295525"/>
-          <a:ext cx="269123" cy="1025525"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="1">
-          <a:noFill/>
-          <a:miter lim="800000"/>
-          <a:headEnd/>
-          <a:tailEnd/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" vert="vert270" wrap="square" lIns="36576" tIns="32004" rIns="36576" bIns="32004" anchor="ctr" upright="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="es-VE" sz="1400" b="1" i="0" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Times New Roman"/>
-              <a:cs typeface="Times New Roman"/>
-            </a:rPr>
-            <a:t>CARGO</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
@@ -2199,19 +2064,19 @@
       <c r="L2" s="8"/>
       <c r="M2" s="8"/>
       <c r="N2" s="8"/>
-      <c r="O2" s="51" t="s">
+      <c r="O2" s="52" t="s">
         <v>4</v>
       </c>
-      <c r="P2" s="52"/>
-      <c r="Q2" s="52"/>
-      <c r="R2" s="52"/>
-      <c r="S2" s="52"/>
-      <c r="T2" s="52"/>
-      <c r="U2" s="52"/>
-      <c r="V2" s="52"/>
-      <c r="W2" s="52"/>
-      <c r="X2" s="52"/>
-      <c r="Y2" s="53"/>
+      <c r="P2" s="53"/>
+      <c r="Q2" s="53"/>
+      <c r="R2" s="53"/>
+      <c r="S2" s="53"/>
+      <c r="T2" s="53"/>
+      <c r="U2" s="53"/>
+      <c r="V2" s="53"/>
+      <c r="W2" s="53"/>
+      <c r="X2" s="53"/>
+      <c r="Y2" s="54"/>
       <c r="Z2" s="1"/>
       <c r="AA2" s="1"/>
       <c r="AB2" s="1"/>
@@ -2233,19 +2098,19 @@
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
       <c r="N3" s="1"/>
-      <c r="O3" s="98" t="s">
+      <c r="O3" s="55" t="s">
         <v>6</v>
       </c>
-      <c r="P3" s="99"/>
-      <c r="Q3" s="99"/>
-      <c r="R3" s="99"/>
-      <c r="S3" s="99"/>
-      <c r="T3" s="99"/>
-      <c r="U3" s="99"/>
-      <c r="V3" s="99"/>
-      <c r="W3" s="99"/>
-      <c r="X3" s="99"/>
-      <c r="Y3" s="100"/>
+      <c r="P3" s="56"/>
+      <c r="Q3" s="56"/>
+      <c r="R3" s="56"/>
+      <c r="S3" s="56"/>
+      <c r="T3" s="56"/>
+      <c r="U3" s="56"/>
+      <c r="V3" s="56"/>
+      <c r="W3" s="56"/>
+      <c r="X3" s="56"/>
+      <c r="Y3" s="57"/>
       <c r="Z3" s="1"/>
       <c r="AA3" s="1"/>
       <c r="AB3" s="1"/>
@@ -2267,19 +2132,19 @@
       <c r="L4" s="18"/>
       <c r="M4" s="18"/>
       <c r="N4" s="18"/>
-      <c r="O4" s="54" t="s">
+      <c r="O4" s="58" t="s">
         <v>8</v>
       </c>
-      <c r="P4" s="55"/>
-      <c r="Q4" s="55"/>
-      <c r="R4" s="55"/>
-      <c r="S4" s="55"/>
-      <c r="T4" s="55"/>
-      <c r="U4" s="55"/>
-      <c r="V4" s="55"/>
-      <c r="W4" s="55"/>
-      <c r="X4" s="55"/>
-      <c r="Y4" s="56"/>
+      <c r="P4" s="59"/>
+      <c r="Q4" s="59"/>
+      <c r="R4" s="59"/>
+      <c r="S4" s="59"/>
+      <c r="T4" s="59"/>
+      <c r="U4" s="59"/>
+      <c r="V4" s="59"/>
+      <c r="W4" s="59"/>
+      <c r="X4" s="59"/>
+      <c r="Y4" s="60"/>
       <c r="Z4" s="1"/>
       <c r="AA4" s="1"/>
       <c r="AB4" s="1"/>
@@ -2328,24 +2193,24 @@
       <c r="E6" s="23">
         <v>4</v>
       </c>
-      <c r="F6" s="57">
+      <c r="F6" s="61">
         <v>5</v>
       </c>
-      <c r="G6" s="58"/>
-      <c r="H6" s="57">
+      <c r="G6" s="62"/>
+      <c r="H6" s="61">
         <v>6</v>
       </c>
-      <c r="I6" s="58"/>
+      <c r="I6" s="62"/>
       <c r="J6" s="23">
         <v>7</v>
       </c>
-      <c r="K6" s="57">
+      <c r="K6" s="61">
         <v>8</v>
       </c>
-      <c r="L6" s="59"/>
-      <c r="M6" s="59"/>
-      <c r="N6" s="59"/>
-      <c r="O6" s="58"/>
+      <c r="L6" s="63"/>
+      <c r="M6" s="63"/>
+      <c r="N6" s="63"/>
+      <c r="O6" s="62"/>
       <c r="P6" s="23">
         <v>9</v>
       </c>
@@ -2381,985 +2246,990 @@
       <c r="AB6" s="24"/>
     </row>
     <row r="7" spans="1:28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="60" t="s">
+      <c r="A7" s="64" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="62" t="s">
+      <c r="B7" s="66" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="64" t="s">
+      <c r="C7" s="68" t="s">
         <v>19</v>
       </c>
-      <c r="D7" s="64"/>
-      <c r="E7" s="66" t="s">
+      <c r="D7" s="68" t="s">
+        <v>50</v>
+      </c>
+      <c r="E7" s="70" t="s">
         <v>20</v>
       </c>
-      <c r="F7" s="76" t="s">
+      <c r="F7" s="80" t="s">
         <v>21</v>
       </c>
-      <c r="G7" s="91"/>
-      <c r="H7" s="76" t="s">
+      <c r="G7" s="97"/>
+      <c r="H7" s="80" t="s">
         <v>22</v>
       </c>
-      <c r="I7" s="77"/>
-      <c r="J7" s="80" t="s">
+      <c r="I7" s="81"/>
+      <c r="J7" s="84" t="s">
         <v>23</v>
       </c>
-      <c r="K7" s="82" t="s">
+      <c r="K7" s="86" t="s">
         <v>24</v>
       </c>
-      <c r="L7" s="83"/>
-      <c r="M7" s="83"/>
-      <c r="N7" s="83"/>
-      <c r="O7" s="84"/>
-      <c r="P7" s="25"/>
-      <c r="Q7" s="70" t="s">
+      <c r="L7" s="87"/>
+      <c r="M7" s="87"/>
+      <c r="N7" s="87"/>
+      <c r="O7" s="88"/>
+      <c r="P7" s="74" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q7" s="74" t="s">
         <v>25</v>
       </c>
-      <c r="R7" s="70" t="s">
+      <c r="R7" s="74" t="s">
         <v>26</v>
       </c>
-      <c r="S7" s="70" t="s">
+      <c r="S7" s="74" t="s">
         <v>27</v>
       </c>
-      <c r="T7" s="70" t="s">
+      <c r="T7" s="74" t="s">
         <v>28</v>
       </c>
-      <c r="U7" s="68" t="s">
+      <c r="U7" s="72" t="s">
         <v>29</v>
       </c>
-      <c r="V7" s="68" t="s">
+      <c r="V7" s="72" t="s">
         <v>30</v>
       </c>
-      <c r="W7" s="70" t="s">
+      <c r="W7" s="74" t="s">
         <v>31</v>
       </c>
-      <c r="X7" s="72" t="s">
+      <c r="X7" s="76" t="s">
         <v>32</v>
       </c>
-      <c r="Y7" s="74" t="s">
+      <c r="Y7" s="78" t="s">
         <v>33</v>
       </c>
-      <c r="Z7" s="26"/>
-      <c r="AA7" s="26"/>
-      <c r="AB7" s="26"/>
+      <c r="Z7" s="25"/>
+      <c r="AA7" s="25"/>
+      <c r="AB7" s="25"/>
     </row>
     <row r="8" spans="1:28" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="61"/>
-      <c r="B8" s="63"/>
-      <c r="C8" s="65"/>
-      <c r="D8" s="65"/>
-      <c r="E8" s="67"/>
-      <c r="F8" s="78"/>
-      <c r="G8" s="92"/>
-      <c r="H8" s="78"/>
-      <c r="I8" s="79"/>
-      <c r="J8" s="81"/>
-      <c r="K8" s="85"/>
-      <c r="L8" s="86"/>
-      <c r="M8" s="86"/>
-      <c r="N8" s="86"/>
-      <c r="O8" s="87"/>
-      <c r="P8" s="27"/>
-      <c r="Q8" s="71"/>
-      <c r="R8" s="71"/>
-      <c r="S8" s="71"/>
-      <c r="T8" s="71"/>
-      <c r="U8" s="69"/>
-      <c r="V8" s="69"/>
-      <c r="W8" s="71"/>
-      <c r="X8" s="73"/>
-      <c r="Y8" s="75"/>
-      <c r="Z8" s="26"/>
-      <c r="AA8" s="26"/>
-      <c r="AB8" s="26"/>
+      <c r="A8" s="65"/>
+      <c r="B8" s="67"/>
+      <c r="C8" s="69"/>
+      <c r="D8" s="69"/>
+      <c r="E8" s="71"/>
+      <c r="F8" s="82"/>
+      <c r="G8" s="98"/>
+      <c r="H8" s="82"/>
+      <c r="I8" s="83"/>
+      <c r="J8" s="85"/>
+      <c r="K8" s="89"/>
+      <c r="L8" s="90"/>
+      <c r="M8" s="90"/>
+      <c r="N8" s="90"/>
+      <c r="O8" s="91"/>
+      <c r="P8" s="94"/>
+      <c r="Q8" s="75"/>
+      <c r="R8" s="75"/>
+      <c r="S8" s="75"/>
+      <c r="T8" s="75"/>
+      <c r="U8" s="73"/>
+      <c r="V8" s="73"/>
+      <c r="W8" s="75"/>
+      <c r="X8" s="77"/>
+      <c r="Y8" s="79"/>
+      <c r="Z8" s="25"/>
+      <c r="AA8" s="25"/>
+      <c r="AB8" s="25"/>
     </row>
     <row r="9" spans="1:28" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="61"/>
-      <c r="B9" s="63"/>
-      <c r="C9" s="65"/>
-      <c r="D9" s="65"/>
-      <c r="E9" s="67"/>
-      <c r="F9" s="80" t="s">
+      <c r="A9" s="65"/>
+      <c r="B9" s="67"/>
+      <c r="C9" s="69"/>
+      <c r="D9" s="69"/>
+      <c r="E9" s="71"/>
+      <c r="F9" s="84" t="s">
         <v>34</v>
       </c>
-      <c r="G9" s="80" t="s">
+      <c r="G9" s="84" t="s">
         <v>35</v>
       </c>
-      <c r="H9" s="60" t="s">
+      <c r="H9" s="64" t="s">
         <v>36</v>
       </c>
-      <c r="I9" s="88" t="s">
+      <c r="I9" s="92" t="s">
         <v>37</v>
       </c>
-      <c r="J9" s="81"/>
-      <c r="K9" s="60" t="s">
+      <c r="J9" s="85"/>
+      <c r="K9" s="64" t="s">
         <v>38</v>
       </c>
-      <c r="L9" s="57" t="s">
+      <c r="L9" s="61" t="s">
         <v>39</v>
       </c>
-      <c r="M9" s="59"/>
-      <c r="N9" s="59"/>
-      <c r="O9" s="58"/>
-      <c r="P9" s="27"/>
-      <c r="Q9" s="71"/>
-      <c r="R9" s="71"/>
-      <c r="S9" s="71"/>
-      <c r="T9" s="71"/>
-      <c r="U9" s="69"/>
-      <c r="V9" s="69"/>
-      <c r="W9" s="71"/>
-      <c r="X9" s="73"/>
-      <c r="Y9" s="75"/>
-      <c r="Z9" s="26"/>
-      <c r="AA9" s="26"/>
-      <c r="AB9" s="26"/>
+      <c r="M9" s="63"/>
+      <c r="N9" s="63"/>
+      <c r="O9" s="62"/>
+      <c r="P9" s="94"/>
+      <c r="Q9" s="75"/>
+      <c r="R9" s="75"/>
+      <c r="S9" s="75"/>
+      <c r="T9" s="75"/>
+      <c r="U9" s="73"/>
+      <c r="V9" s="73"/>
+      <c r="W9" s="75"/>
+      <c r="X9" s="77"/>
+      <c r="Y9" s="79"/>
+      <c r="Z9" s="25"/>
+      <c r="AA9" s="25"/>
+      <c r="AB9" s="25"/>
     </row>
     <row r="10" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="61"/>
-      <c r="B10" s="63"/>
-      <c r="C10" s="65"/>
-      <c r="D10" s="65"/>
-      <c r="E10" s="67"/>
-      <c r="F10" s="81"/>
-      <c r="G10" s="81"/>
-      <c r="H10" s="61"/>
-      <c r="I10" s="89"/>
-      <c r="J10" s="81"/>
-      <c r="K10" s="61"/>
-      <c r="L10" s="28" t="s">
+      <c r="A10" s="65"/>
+      <c r="B10" s="67"/>
+      <c r="C10" s="69"/>
+      <c r="D10" s="69"/>
+      <c r="E10" s="71"/>
+      <c r="F10" s="85"/>
+      <c r="G10" s="85"/>
+      <c r="H10" s="65"/>
+      <c r="I10" s="93"/>
+      <c r="J10" s="85"/>
+      <c r="K10" s="65"/>
+      <c r="L10" s="26" t="s">
         <v>40</v>
       </c>
-      <c r="M10" s="28" t="s">
+      <c r="M10" s="26" t="s">
         <v>41</v>
       </c>
-      <c r="N10" s="28" t="s">
+      <c r="N10" s="26" t="s">
         <v>42</v>
       </c>
-      <c r="O10" s="28" t="s">
+      <c r="O10" s="26" t="s">
         <v>43</v>
       </c>
-      <c r="P10" s="27"/>
-      <c r="Q10" s="71"/>
-      <c r="R10" s="71"/>
-      <c r="S10" s="71"/>
-      <c r="T10" s="71"/>
-      <c r="U10" s="69"/>
-      <c r="V10" s="69"/>
-      <c r="W10" s="71"/>
-      <c r="X10" s="73"/>
-      <c r="Y10" s="75"/>
-      <c r="Z10" s="26"/>
-      <c r="AA10" s="26"/>
-      <c r="AB10" s="26"/>
+      <c r="P10" s="95"/>
+      <c r="Q10" s="75"/>
+      <c r="R10" s="75"/>
+      <c r="S10" s="75"/>
+      <c r="T10" s="75"/>
+      <c r="U10" s="73"/>
+      <c r="V10" s="73"/>
+      <c r="W10" s="75"/>
+      <c r="X10" s="77"/>
+      <c r="Y10" s="79"/>
+      <c r="Z10" s="25"/>
+      <c r="AA10" s="25"/>
+      <c r="AB10" s="25"/>
     </row>
     <row r="11" spans="1:28" ht="48" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="29"/>
-      <c r="B11" s="29"/>
-      <c r="C11" s="29"/>
-      <c r="D11" s="29"/>
-      <c r="E11" s="29"/>
-      <c r="F11" s="29"/>
-      <c r="G11" s="29"/>
-      <c r="H11" s="30"/>
-      <c r="I11" s="29"/>
-      <c r="J11" s="30"/>
-      <c r="K11" s="31"/>
-      <c r="L11" s="32"/>
-      <c r="M11" s="29"/>
-      <c r="N11" s="29"/>
-      <c r="O11" s="29"/>
-      <c r="P11" s="29"/>
-      <c r="Q11" s="33"/>
-      <c r="R11" s="33"/>
-      <c r="S11" s="33"/>
-      <c r="T11" s="33"/>
-      <c r="U11" s="33"/>
-      <c r="V11" s="33"/>
-      <c r="W11" s="33"/>
-      <c r="X11" s="33"/>
-      <c r="Y11" s="33"/>
-      <c r="Z11" s="26"/>
-      <c r="AA11" s="26"/>
-      <c r="AB11" s="26"/>
+      <c r="A11" s="27"/>
+      <c r="B11" s="27"/>
+      <c r="C11" s="27"/>
+      <c r="D11" s="27"/>
+      <c r="E11" s="27"/>
+      <c r="F11" s="27"/>
+      <c r="G11" s="27"/>
+      <c r="H11" s="28"/>
+      <c r="I11" s="27"/>
+      <c r="J11" s="28"/>
+      <c r="K11" s="29"/>
+      <c r="L11" s="30"/>
+      <c r="M11" s="27"/>
+      <c r="N11" s="27"/>
+      <c r="O11" s="27"/>
+      <c r="P11" s="27"/>
+      <c r="Q11" s="31"/>
+      <c r="R11" s="31"/>
+      <c r="S11" s="31"/>
+      <c r="T11" s="31"/>
+      <c r="U11" s="31"/>
+      <c r="V11" s="31"/>
+      <c r="W11" s="31"/>
+      <c r="X11" s="31"/>
+      <c r="Y11" s="31"/>
+      <c r="Z11" s="25"/>
+      <c r="AA11" s="25"/>
+      <c r="AB11" s="25"/>
     </row>
     <row r="12" spans="1:28" ht="48" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="29"/>
-      <c r="B12" s="29"/>
-      <c r="C12" s="29"/>
-      <c r="D12" s="29"/>
-      <c r="E12" s="29"/>
-      <c r="F12" s="29"/>
-      <c r="G12" s="29"/>
-      <c r="H12" s="30"/>
-      <c r="I12" s="29"/>
-      <c r="J12" s="30"/>
-      <c r="K12" s="31"/>
-      <c r="L12" s="32"/>
-      <c r="M12" s="29"/>
-      <c r="N12" s="29"/>
-      <c r="O12" s="29"/>
-      <c r="P12" s="29"/>
-      <c r="Q12" s="33"/>
-      <c r="R12" s="33"/>
-      <c r="S12" s="33"/>
-      <c r="T12" s="33"/>
-      <c r="U12" s="33"/>
-      <c r="V12" s="33"/>
-      <c r="W12" s="33"/>
-      <c r="X12" s="33"/>
-      <c r="Y12" s="33"/>
-      <c r="Z12" s="26"/>
-      <c r="AA12" s="26"/>
-      <c r="AB12" s="26"/>
+      <c r="A12" s="27"/>
+      <c r="B12" s="27"/>
+      <c r="C12" s="27"/>
+      <c r="D12" s="27"/>
+      <c r="E12" s="27"/>
+      <c r="F12" s="27"/>
+      <c r="G12" s="27"/>
+      <c r="H12" s="28"/>
+      <c r="I12" s="27"/>
+      <c r="J12" s="28"/>
+      <c r="K12" s="29"/>
+      <c r="L12" s="30"/>
+      <c r="M12" s="27"/>
+      <c r="N12" s="27"/>
+      <c r="O12" s="27"/>
+      <c r="P12" s="27"/>
+      <c r="Q12" s="31"/>
+      <c r="R12" s="31"/>
+      <c r="S12" s="31"/>
+      <c r="T12" s="31"/>
+      <c r="U12" s="31"/>
+      <c r="V12" s="31"/>
+      <c r="W12" s="31"/>
+      <c r="X12" s="31"/>
+      <c r="Y12" s="31"/>
+      <c r="Z12" s="25"/>
+      <c r="AA12" s="25"/>
+      <c r="AB12" s="25"/>
     </row>
     <row r="13" spans="1:28" ht="48" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="29"/>
-      <c r="B13" s="29"/>
-      <c r="C13" s="29"/>
-      <c r="D13" s="29"/>
-      <c r="E13" s="29"/>
-      <c r="F13" s="29"/>
-      <c r="G13" s="29"/>
-      <c r="H13" s="30"/>
-      <c r="I13" s="29"/>
-      <c r="J13" s="30"/>
-      <c r="K13" s="31"/>
-      <c r="L13" s="29"/>
-      <c r="M13" s="29"/>
-      <c r="N13" s="29"/>
-      <c r="O13" s="29"/>
-      <c r="P13" s="29"/>
-      <c r="Q13" s="33"/>
-      <c r="R13" s="33"/>
-      <c r="S13" s="33"/>
-      <c r="T13" s="33"/>
-      <c r="U13" s="33"/>
-      <c r="V13" s="33"/>
-      <c r="W13" s="33"/>
-      <c r="X13" s="33"/>
-      <c r="Y13" s="33"/>
-      <c r="Z13" s="26"/>
-      <c r="AA13" s="26"/>
-      <c r="AB13" s="26"/>
+      <c r="A13" s="27"/>
+      <c r="B13" s="27"/>
+      <c r="C13" s="27"/>
+      <c r="D13" s="27"/>
+      <c r="E13" s="27"/>
+      <c r="F13" s="27"/>
+      <c r="G13" s="27"/>
+      <c r="H13" s="28"/>
+      <c r="I13" s="27"/>
+      <c r="J13" s="28"/>
+      <c r="K13" s="29"/>
+      <c r="L13" s="27"/>
+      <c r="M13" s="27"/>
+      <c r="N13" s="27"/>
+      <c r="O13" s="27"/>
+      <c r="P13" s="27"/>
+      <c r="Q13" s="31"/>
+      <c r="R13" s="31"/>
+      <c r="S13" s="31"/>
+      <c r="T13" s="31"/>
+      <c r="U13" s="31"/>
+      <c r="V13" s="31"/>
+      <c r="W13" s="31"/>
+      <c r="X13" s="31"/>
+      <c r="Y13" s="31"/>
+      <c r="Z13" s="25"/>
+      <c r="AA13" s="25"/>
+      <c r="AB13" s="25"/>
     </row>
     <row r="14" spans="1:28" ht="48" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="29"/>
-      <c r="B14" s="29"/>
-      <c r="C14" s="29"/>
-      <c r="D14" s="29"/>
-      <c r="E14" s="29"/>
-      <c r="F14" s="29"/>
-      <c r="G14" s="29"/>
-      <c r="H14" s="30"/>
-      <c r="I14" s="29"/>
-      <c r="J14" s="30"/>
-      <c r="K14" s="31"/>
-      <c r="L14" s="32"/>
-      <c r="M14" s="29"/>
-      <c r="N14" s="29"/>
-      <c r="O14" s="29"/>
-      <c r="P14" s="29"/>
-      <c r="Q14" s="33"/>
-      <c r="R14" s="33"/>
-      <c r="S14" s="33"/>
-      <c r="T14" s="33"/>
-      <c r="U14" s="33"/>
-      <c r="V14" s="33"/>
-      <c r="W14" s="33"/>
-      <c r="X14" s="33"/>
-      <c r="Y14" s="33"/>
-      <c r="Z14" s="26"/>
-      <c r="AA14" s="26"/>
-      <c r="AB14" s="26"/>
+      <c r="A14" s="27"/>
+      <c r="B14" s="27"/>
+      <c r="C14" s="27"/>
+      <c r="D14" s="27"/>
+      <c r="E14" s="27"/>
+      <c r="F14" s="27"/>
+      <c r="G14" s="27"/>
+      <c r="H14" s="28"/>
+      <c r="I14" s="27"/>
+      <c r="J14" s="28"/>
+      <c r="K14" s="29"/>
+      <c r="L14" s="30"/>
+      <c r="M14" s="27"/>
+      <c r="N14" s="27"/>
+      <c r="O14" s="27"/>
+      <c r="P14" s="27"/>
+      <c r="Q14" s="31"/>
+      <c r="R14" s="31"/>
+      <c r="S14" s="46"/>
+      <c r="T14" s="31"/>
+      <c r="U14" s="31"/>
+      <c r="V14" s="31"/>
+      <c r="W14" s="31"/>
+      <c r="X14" s="31"/>
+      <c r="Y14" s="31"/>
+      <c r="Z14" s="25"/>
+      <c r="AA14" s="25"/>
+      <c r="AB14" s="25"/>
     </row>
     <row r="15" spans="1:28" ht="48" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="29"/>
-      <c r="B15" s="29"/>
-      <c r="C15" s="29"/>
-      <c r="D15" s="29"/>
-      <c r="E15" s="29"/>
-      <c r="F15" s="29"/>
-      <c r="G15" s="29"/>
-      <c r="H15" s="30"/>
-      <c r="I15" s="29"/>
-      <c r="J15" s="30"/>
-      <c r="K15" s="31"/>
-      <c r="L15" s="32"/>
-      <c r="M15" s="29"/>
-      <c r="N15" s="29"/>
-      <c r="O15" s="29"/>
-      <c r="P15" s="29"/>
-      <c r="Q15" s="33"/>
-      <c r="R15" s="33"/>
-      <c r="S15" s="33"/>
-      <c r="T15" s="48"/>
-      <c r="U15" s="33"/>
-      <c r="V15" s="33"/>
-      <c r="W15" s="33"/>
-      <c r="X15" s="33"/>
-      <c r="Y15" s="33"/>
-      <c r="Z15" s="26"/>
-      <c r="AA15" s="26"/>
-      <c r="AB15" s="26"/>
+      <c r="A15" s="27"/>
+      <c r="B15" s="27"/>
+      <c r="C15" s="27"/>
+      <c r="D15" s="27"/>
+      <c r="E15" s="27"/>
+      <c r="F15" s="27"/>
+      <c r="G15" s="27"/>
+      <c r="H15" s="28"/>
+      <c r="I15" s="27"/>
+      <c r="J15" s="28"/>
+      <c r="K15" s="29"/>
+      <c r="L15" s="30"/>
+      <c r="M15" s="27"/>
+      <c r="N15" s="27"/>
+      <c r="O15" s="27"/>
+      <c r="P15" s="27"/>
+      <c r="Q15" s="31"/>
+      <c r="R15" s="31"/>
+      <c r="S15" s="31"/>
+      <c r="T15" s="46"/>
+      <c r="U15" s="31"/>
+      <c r="V15" s="31"/>
+      <c r="W15" s="31"/>
+      <c r="X15" s="31"/>
+      <c r="Y15" s="31"/>
+      <c r="Z15" s="25"/>
+      <c r="AA15" s="25"/>
+      <c r="AB15" s="25"/>
     </row>
     <row r="16" spans="1:28" ht="48" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="93"/>
-      <c r="B16" s="93"/>
-      <c r="C16" s="93"/>
-      <c r="D16" s="93"/>
-      <c r="E16" s="93"/>
-      <c r="F16" s="93"/>
-      <c r="G16" s="93"/>
-      <c r="H16" s="94"/>
-      <c r="I16" s="93"/>
-      <c r="J16" s="94"/>
-      <c r="K16" s="95"/>
-      <c r="L16" s="96"/>
-      <c r="M16" s="93"/>
-      <c r="N16" s="93"/>
-      <c r="O16" s="93"/>
-      <c r="P16" s="93"/>
-      <c r="Q16" s="97"/>
-      <c r="R16" s="97"/>
-      <c r="S16" s="97"/>
-      <c r="T16" s="97"/>
-      <c r="U16" s="97"/>
-      <c r="V16" s="97"/>
-      <c r="W16" s="97"/>
-      <c r="X16" s="97"/>
-      <c r="Y16" s="97"/>
-      <c r="Z16" s="26"/>
-      <c r="AA16" s="26"/>
-      <c r="AB16" s="26"/>
+      <c r="A16" s="49"/>
+      <c r="B16" s="49"/>
+      <c r="C16" s="49"/>
+      <c r="D16" s="49"/>
+      <c r="E16" s="49"/>
+      <c r="F16" s="49"/>
+      <c r="G16" s="49"/>
+      <c r="H16" s="50"/>
+      <c r="I16" s="49"/>
+      <c r="J16" s="50"/>
+      <c r="K16" s="29"/>
+      <c r="L16" s="30"/>
+      <c r="M16" s="49"/>
+      <c r="N16" s="49"/>
+      <c r="O16" s="49"/>
+      <c r="P16" s="49"/>
+      <c r="Q16" s="51"/>
+      <c r="R16" s="51"/>
+      <c r="S16" s="51"/>
+      <c r="T16" s="51"/>
+      <c r="U16" s="51"/>
+      <c r="V16" s="51"/>
+      <c r="W16" s="51"/>
+      <c r="X16" s="51"/>
+      <c r="Y16" s="51"/>
+      <c r="Z16" s="25"/>
+      <c r="AA16" s="25"/>
+      <c r="AB16" s="25"/>
     </row>
     <row r="17" spans="1:28" ht="48" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="93"/>
-      <c r="B17" s="93"/>
-      <c r="C17" s="93"/>
-      <c r="D17" s="93"/>
-      <c r="E17" s="93"/>
-      <c r="F17" s="93"/>
-      <c r="G17" s="93"/>
-      <c r="H17" s="94"/>
-      <c r="I17" s="93"/>
-      <c r="J17" s="94"/>
-      <c r="K17" s="95"/>
-      <c r="L17" s="96"/>
-      <c r="M17" s="93"/>
-      <c r="N17" s="93"/>
-      <c r="O17" s="93"/>
-      <c r="P17" s="93"/>
-      <c r="Q17" s="97"/>
-      <c r="R17" s="97"/>
-      <c r="S17" s="97"/>
-      <c r="T17" s="97"/>
-      <c r="U17" s="97"/>
-      <c r="V17" s="97"/>
-      <c r="W17" s="97"/>
-      <c r="X17" s="97"/>
-      <c r="Y17" s="97"/>
-      <c r="Z17" s="26"/>
-      <c r="AA17" s="26"/>
-      <c r="AB17" s="26"/>
+      <c r="A17" s="49"/>
+      <c r="B17" s="49"/>
+      <c r="C17" s="49"/>
+      <c r="D17" s="49"/>
+      <c r="E17" s="49"/>
+      <c r="F17" s="49"/>
+      <c r="G17" s="49"/>
+      <c r="H17" s="50"/>
+      <c r="I17" s="49"/>
+      <c r="J17" s="50"/>
+      <c r="K17" s="29"/>
+      <c r="L17" s="30"/>
+      <c r="M17" s="49"/>
+      <c r="N17" s="49"/>
+      <c r="O17" s="49"/>
+      <c r="P17" s="49"/>
+      <c r="Q17" s="51"/>
+      <c r="R17" s="51"/>
+      <c r="S17" s="51"/>
+      <c r="T17" s="51"/>
+      <c r="U17" s="51"/>
+      <c r="V17" s="51"/>
+      <c r="W17" s="51"/>
+      <c r="X17" s="51"/>
+      <c r="Y17" s="51"/>
+      <c r="Z17" s="25"/>
+      <c r="AA17" s="25"/>
+      <c r="AB17" s="25"/>
     </row>
     <row r="18" spans="1:28" ht="48" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="93"/>
-      <c r="B18" s="93"/>
-      <c r="C18" s="93"/>
-      <c r="D18" s="93"/>
-      <c r="E18" s="93"/>
-      <c r="F18" s="93"/>
-      <c r="G18" s="93"/>
-      <c r="H18" s="30"/>
-      <c r="I18" s="29"/>
-      <c r="J18" s="30"/>
-      <c r="K18" s="31"/>
-      <c r="L18" s="29"/>
-      <c r="M18" s="29"/>
-      <c r="N18" s="29"/>
-      <c r="O18" s="29"/>
-      <c r="P18" s="29"/>
-      <c r="Q18" s="33"/>
-      <c r="R18" s="33"/>
-      <c r="S18" s="33"/>
-      <c r="T18" s="33"/>
-      <c r="U18" s="33"/>
-      <c r="V18" s="33"/>
-      <c r="W18" s="33"/>
-      <c r="X18" s="33"/>
-      <c r="Y18" s="33"/>
-      <c r="Z18" s="26"/>
-      <c r="AA18" s="26"/>
-      <c r="AB18" s="26"/>
+      <c r="A18" s="49"/>
+      <c r="B18" s="49"/>
+      <c r="C18" s="49"/>
+      <c r="D18" s="49"/>
+      <c r="E18" s="49"/>
+      <c r="F18" s="49"/>
+      <c r="G18" s="49"/>
+      <c r="H18" s="28"/>
+      <c r="I18" s="27"/>
+      <c r="J18" s="28"/>
+      <c r="K18" s="29"/>
+      <c r="L18" s="27"/>
+      <c r="M18" s="27"/>
+      <c r="N18" s="27"/>
+      <c r="O18" s="27"/>
+      <c r="P18" s="27"/>
+      <c r="Q18" s="31"/>
+      <c r="R18" s="31"/>
+      <c r="S18" s="31"/>
+      <c r="T18" s="31"/>
+      <c r="U18" s="31"/>
+      <c r="V18" s="31"/>
+      <c r="W18" s="31"/>
+      <c r="X18" s="31"/>
+      <c r="Y18" s="31"/>
+      <c r="Z18" s="25"/>
+      <c r="AA18" s="25"/>
+      <c r="AB18" s="25"/>
     </row>
     <row r="19" spans="1:28" ht="48" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="93"/>
-      <c r="B19" s="93"/>
-      <c r="C19" s="93"/>
-      <c r="D19" s="93"/>
-      <c r="E19" s="93"/>
-      <c r="F19" s="93"/>
-      <c r="G19" s="93"/>
-      <c r="H19" s="30"/>
-      <c r="I19" s="29"/>
-      <c r="J19" s="30"/>
-      <c r="K19" s="31"/>
-      <c r="L19" s="32"/>
-      <c r="M19" s="29"/>
-      <c r="N19" s="29"/>
-      <c r="O19" s="29"/>
-      <c r="P19" s="29"/>
-      <c r="Q19" s="33"/>
-      <c r="R19" s="33"/>
-      <c r="S19" s="33"/>
-      <c r="T19" s="33"/>
-      <c r="U19" s="33"/>
-      <c r="V19" s="33"/>
-      <c r="W19" s="33"/>
-      <c r="X19" s="33"/>
-      <c r="Y19" s="33"/>
-      <c r="Z19" s="26"/>
-      <c r="AA19" s="26"/>
-      <c r="AB19" s="26"/>
+      <c r="A19" s="49"/>
+      <c r="B19" s="49"/>
+      <c r="C19" s="49"/>
+      <c r="D19" s="49"/>
+      <c r="E19" s="49"/>
+      <c r="F19" s="49"/>
+      <c r="G19" s="49"/>
+      <c r="H19" s="28"/>
+      <c r="I19" s="27"/>
+      <c r="J19" s="28"/>
+      <c r="K19" s="29"/>
+      <c r="L19" s="30"/>
+      <c r="M19" s="27"/>
+      <c r="N19" s="27"/>
+      <c r="O19" s="27"/>
+      <c r="P19" s="27"/>
+      <c r="Q19" s="31"/>
+      <c r="R19" s="31"/>
+      <c r="S19" s="31"/>
+      <c r="T19" s="31"/>
+      <c r="U19" s="31"/>
+      <c r="V19" s="31"/>
+      <c r="W19" s="31"/>
+      <c r="X19" s="31"/>
+      <c r="Y19" s="31"/>
+      <c r="Z19" s="25"/>
+      <c r="AA19" s="25"/>
+      <c r="AB19" s="25"/>
     </row>
     <row r="20" spans="1:28" ht="48" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="93"/>
-      <c r="B20" s="93"/>
-      <c r="C20" s="93"/>
-      <c r="D20" s="93"/>
-      <c r="E20" s="93"/>
-      <c r="F20" s="93"/>
-      <c r="G20" s="93"/>
-      <c r="H20" s="30"/>
-      <c r="I20" s="29"/>
-      <c r="J20" s="30"/>
-      <c r="K20" s="31"/>
-      <c r="L20" s="32"/>
-      <c r="M20" s="29"/>
-      <c r="N20" s="29"/>
-      <c r="O20" s="29"/>
-      <c r="P20" s="29"/>
-      <c r="Q20" s="33"/>
-      <c r="R20" s="33"/>
-      <c r="S20" s="33"/>
-      <c r="T20" s="48"/>
-      <c r="U20" s="33"/>
-      <c r="V20" s="33"/>
-      <c r="W20" s="33"/>
-      <c r="X20" s="33"/>
-      <c r="Y20" s="33"/>
-      <c r="Z20" s="26"/>
-      <c r="AA20" s="26"/>
-      <c r="AB20" s="26"/>
+      <c r="A20" s="49"/>
+      <c r="B20" s="49"/>
+      <c r="C20" s="49"/>
+      <c r="D20" s="49"/>
+      <c r="E20" s="49"/>
+      <c r="F20" s="49"/>
+      <c r="G20" s="49"/>
+      <c r="H20" s="28"/>
+      <c r="I20" s="27"/>
+      <c r="J20" s="28"/>
+      <c r="K20" s="29"/>
+      <c r="L20" s="30"/>
+      <c r="M20" s="27"/>
+      <c r="N20" s="27"/>
+      <c r="O20" s="27"/>
+      <c r="P20" s="27"/>
+      <c r="Q20" s="31"/>
+      <c r="R20" s="31"/>
+      <c r="S20" s="31"/>
+      <c r="T20" s="46"/>
+      <c r="U20" s="31"/>
+      <c r="V20" s="31"/>
+      <c r="W20" s="31"/>
+      <c r="X20" s="31"/>
+      <c r="Y20" s="31"/>
+      <c r="Z20" s="25"/>
+      <c r="AA20" s="25"/>
+      <c r="AB20" s="25"/>
     </row>
     <row r="21" spans="1:28" ht="48" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="93"/>
-      <c r="B21" s="93"/>
-      <c r="C21" s="93"/>
-      <c r="D21" s="93"/>
-      <c r="E21" s="93"/>
-      <c r="F21" s="93"/>
-      <c r="G21" s="93"/>
-      <c r="H21" s="30"/>
-      <c r="I21" s="29"/>
-      <c r="J21" s="30"/>
-      <c r="K21" s="31"/>
-      <c r="L21" s="32"/>
-      <c r="M21" s="29"/>
-      <c r="N21" s="29"/>
-      <c r="O21" s="29"/>
-      <c r="P21" s="29"/>
-      <c r="Q21" s="33"/>
-      <c r="R21" s="33"/>
-      <c r="S21" s="33"/>
-      <c r="T21" s="33"/>
-      <c r="U21" s="33"/>
-      <c r="V21" s="33"/>
-      <c r="W21" s="33"/>
-      <c r="X21" s="33"/>
-      <c r="Y21" s="33"/>
-      <c r="Z21" s="26"/>
-      <c r="AA21" s="26"/>
-      <c r="AB21" s="26"/>
+      <c r="A21" s="49"/>
+      <c r="B21" s="49"/>
+      <c r="C21" s="49"/>
+      <c r="D21" s="49"/>
+      <c r="E21" s="49"/>
+      <c r="F21" s="49"/>
+      <c r="G21" s="49"/>
+      <c r="H21" s="28"/>
+      <c r="I21" s="27"/>
+      <c r="J21" s="28"/>
+      <c r="K21" s="29"/>
+      <c r="L21" s="30"/>
+      <c r="M21" s="27"/>
+      <c r="N21" s="27"/>
+      <c r="O21" s="27"/>
+      <c r="P21" s="27"/>
+      <c r="Q21" s="31"/>
+      <c r="R21" s="31"/>
+      <c r="S21" s="31"/>
+      <c r="T21" s="31"/>
+      <c r="U21" s="31"/>
+      <c r="V21" s="31"/>
+      <c r="W21" s="31"/>
+      <c r="X21" s="31"/>
+      <c r="Y21" s="31"/>
+      <c r="Z21" s="25"/>
+      <c r="AA21" s="25"/>
+      <c r="AB21" s="25"/>
     </row>
     <row r="22" spans="1:28" ht="48" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="93"/>
-      <c r="B22" s="93"/>
-      <c r="C22" s="93"/>
-      <c r="D22" s="93"/>
-      <c r="E22" s="93"/>
-      <c r="F22" s="93"/>
-      <c r="G22" s="93"/>
-      <c r="H22" s="30"/>
-      <c r="I22" s="29"/>
-      <c r="J22" s="30"/>
-      <c r="K22" s="31"/>
-      <c r="L22" s="32"/>
-      <c r="M22" s="29"/>
-      <c r="N22" s="29"/>
-      <c r="O22" s="29"/>
-      <c r="P22" s="29"/>
-      <c r="Q22" s="33"/>
-      <c r="R22" s="33"/>
-      <c r="S22" s="33"/>
-      <c r="T22" s="33"/>
-      <c r="U22" s="33"/>
-      <c r="V22" s="33"/>
-      <c r="W22" s="33"/>
-      <c r="X22" s="33"/>
-      <c r="Y22" s="33"/>
-      <c r="Z22" s="26"/>
-      <c r="AA22" s="26"/>
-      <c r="AB22" s="26"/>
+      <c r="A22" s="49"/>
+      <c r="B22" s="49"/>
+      <c r="C22" s="49"/>
+      <c r="D22" s="49"/>
+      <c r="E22" s="49"/>
+      <c r="F22" s="49"/>
+      <c r="G22" s="49"/>
+      <c r="H22" s="28"/>
+      <c r="I22" s="27"/>
+      <c r="J22" s="28"/>
+      <c r="K22" s="29"/>
+      <c r="L22" s="30"/>
+      <c r="M22" s="27"/>
+      <c r="N22" s="27"/>
+      <c r="O22" s="27"/>
+      <c r="P22" s="27"/>
+      <c r="Q22" s="31"/>
+      <c r="R22" s="31"/>
+      <c r="S22" s="31"/>
+      <c r="T22" s="31"/>
+      <c r="U22" s="31"/>
+      <c r="V22" s="31"/>
+      <c r="W22" s="31"/>
+      <c r="X22" s="31"/>
+      <c r="Y22" s="31"/>
+      <c r="Z22" s="25"/>
+      <c r="AA22" s="25"/>
+      <c r="AB22" s="25"/>
     </row>
     <row r="23" spans="1:28" ht="48" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="93"/>
-      <c r="B23" s="93"/>
-      <c r="C23" s="93"/>
-      <c r="D23" s="93"/>
-      <c r="E23" s="93"/>
-      <c r="F23" s="93"/>
-      <c r="G23" s="93"/>
-      <c r="H23" s="30"/>
-      <c r="I23" s="29"/>
-      <c r="J23" s="30"/>
-      <c r="K23" s="31"/>
-      <c r="L23" s="29"/>
-      <c r="M23" s="29"/>
-      <c r="N23" s="29"/>
-      <c r="O23" s="29"/>
-      <c r="P23" s="29"/>
-      <c r="Q23" s="33"/>
-      <c r="R23" s="33"/>
-      <c r="S23" s="33"/>
-      <c r="T23" s="33"/>
-      <c r="U23" s="33"/>
-      <c r="V23" s="33"/>
-      <c r="W23" s="33"/>
-      <c r="X23" s="33"/>
-      <c r="Y23" s="33"/>
-      <c r="Z23" s="26"/>
-      <c r="AA23" s="26"/>
-      <c r="AB23" s="26"/>
+      <c r="A23" s="49"/>
+      <c r="B23" s="49"/>
+      <c r="C23" s="49"/>
+      <c r="D23" s="49"/>
+      <c r="E23" s="49"/>
+      <c r="F23" s="49"/>
+      <c r="G23" s="49"/>
+      <c r="H23" s="28"/>
+      <c r="I23" s="27"/>
+      <c r="J23" s="28"/>
+      <c r="K23" s="29"/>
+      <c r="L23" s="27"/>
+      <c r="M23" s="27"/>
+      <c r="N23" s="27"/>
+      <c r="O23" s="27"/>
+      <c r="P23" s="27"/>
+      <c r="Q23" s="31"/>
+      <c r="R23" s="31"/>
+      <c r="S23" s="31"/>
+      <c r="T23" s="31"/>
+      <c r="U23" s="31"/>
+      <c r="V23" s="31"/>
+      <c r="W23" s="31"/>
+      <c r="X23" s="31"/>
+      <c r="Y23" s="31"/>
+      <c r="Z23" s="25"/>
+      <c r="AA23" s="25"/>
+      <c r="AB23" s="25"/>
     </row>
     <row r="24" spans="1:28" ht="48" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="93"/>
-      <c r="B24" s="93"/>
-      <c r="C24" s="93"/>
-      <c r="D24" s="93"/>
-      <c r="E24" s="93"/>
-      <c r="F24" s="93"/>
-      <c r="G24" s="93"/>
-      <c r="H24" s="30"/>
-      <c r="I24" s="29"/>
-      <c r="J24" s="30"/>
-      <c r="K24" s="31"/>
-      <c r="L24" s="32"/>
-      <c r="M24" s="29"/>
-      <c r="N24" s="29"/>
-      <c r="O24" s="29"/>
-      <c r="P24" s="29"/>
-      <c r="Q24" s="33"/>
-      <c r="R24" s="33"/>
-      <c r="S24" s="33"/>
-      <c r="T24" s="33"/>
-      <c r="U24" s="33"/>
-      <c r="V24" s="33"/>
-      <c r="W24" s="33"/>
-      <c r="X24" s="33"/>
-      <c r="Y24" s="33"/>
-      <c r="Z24" s="26"/>
-      <c r="AA24" s="26"/>
-      <c r="AB24" s="26"/>
+      <c r="A24" s="49"/>
+      <c r="B24" s="49"/>
+      <c r="C24" s="49"/>
+      <c r="D24" s="49"/>
+      <c r="E24" s="49"/>
+      <c r="F24" s="49"/>
+      <c r="G24" s="49"/>
+      <c r="H24" s="28"/>
+      <c r="I24" s="27"/>
+      <c r="J24" s="28"/>
+      <c r="K24" s="29"/>
+      <c r="L24" s="30"/>
+      <c r="M24" s="27"/>
+      <c r="N24" s="27"/>
+      <c r="O24" s="27"/>
+      <c r="P24" s="27"/>
+      <c r="Q24" s="31"/>
+      <c r="R24" s="31"/>
+      <c r="S24" s="31"/>
+      <c r="T24" s="31"/>
+      <c r="U24" s="31"/>
+      <c r="V24" s="31"/>
+      <c r="W24" s="31"/>
+      <c r="X24" s="31"/>
+      <c r="Y24" s="31"/>
+      <c r="Z24" s="25"/>
+      <c r="AA24" s="25"/>
+      <c r="AB24" s="25"/>
     </row>
     <row r="25" spans="1:28" ht="48" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="93"/>
-      <c r="B25" s="93"/>
-      <c r="C25" s="93"/>
-      <c r="D25" s="93"/>
-      <c r="E25" s="93"/>
-      <c r="F25" s="93"/>
-      <c r="G25" s="93"/>
-      <c r="H25" s="30"/>
-      <c r="I25" s="29"/>
-      <c r="J25" s="30"/>
-      <c r="K25" s="31"/>
-      <c r="L25" s="32"/>
-      <c r="M25" s="29"/>
-      <c r="N25" s="29"/>
-      <c r="O25" s="29"/>
-      <c r="P25" s="29"/>
-      <c r="Q25" s="33"/>
-      <c r="R25" s="33"/>
-      <c r="T25" s="48"/>
-      <c r="U25" s="33"/>
-      <c r="V25" s="33"/>
-      <c r="W25" s="33"/>
-      <c r="X25" s="33"/>
-      <c r="Y25" s="33"/>
-      <c r="Z25" s="26"/>
-      <c r="AA25" s="26"/>
-      <c r="AB25" s="26"/>
+      <c r="A25" s="49"/>
+      <c r="B25" s="49"/>
+      <c r="C25" s="49"/>
+      <c r="D25" s="49"/>
+      <c r="E25" s="49"/>
+      <c r="F25" s="49"/>
+      <c r="G25" s="49"/>
+      <c r="H25" s="28"/>
+      <c r="I25" s="27"/>
+      <c r="J25" s="28"/>
+      <c r="K25" s="29"/>
+      <c r="L25" s="30"/>
+      <c r="M25" s="27"/>
+      <c r="N25" s="27"/>
+      <c r="O25" s="27"/>
+      <c r="P25" s="27"/>
+      <c r="Q25" s="31"/>
+      <c r="R25" s="31"/>
+      <c r="S25" s="31"/>
+      <c r="T25" s="46"/>
+      <c r="U25" s="31"/>
+      <c r="V25" s="31"/>
+      <c r="W25" s="31"/>
+      <c r="X25" s="31"/>
+      <c r="Y25" s="31"/>
+      <c r="Z25" s="25"/>
+      <c r="AA25" s="25"/>
+      <c r="AB25" s="25"/>
     </row>
     <row r="26" spans="1:28" ht="48" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="93"/>
-      <c r="B26" s="93"/>
-      <c r="C26" s="93"/>
-      <c r="D26" s="93"/>
-      <c r="E26" s="93"/>
-      <c r="F26" s="93"/>
-      <c r="G26" s="93"/>
-      <c r="H26" s="30"/>
-      <c r="I26" s="29"/>
-      <c r="J26" s="30"/>
-      <c r="K26" s="31"/>
-      <c r="L26" s="32"/>
-      <c r="M26" s="29"/>
-      <c r="N26" s="29"/>
-      <c r="O26" s="29"/>
-      <c r="P26" s="29"/>
-      <c r="Q26" s="33"/>
-      <c r="R26" s="33"/>
-      <c r="S26" s="33"/>
-      <c r="T26" s="48"/>
-      <c r="U26" s="33"/>
-      <c r="V26" s="33"/>
-      <c r="W26" s="33"/>
-      <c r="X26" s="33"/>
-      <c r="Y26" s="33"/>
-      <c r="Z26" s="26"/>
-      <c r="AA26" s="26"/>
-      <c r="AB26" s="26"/>
+      <c r="A26" s="49"/>
+      <c r="B26" s="49"/>
+      <c r="C26" s="49"/>
+      <c r="D26" s="49"/>
+      <c r="E26" s="49"/>
+      <c r="F26" s="49"/>
+      <c r="G26" s="49"/>
+      <c r="H26" s="28"/>
+      <c r="I26" s="27"/>
+      <c r="J26" s="28"/>
+      <c r="K26" s="29"/>
+      <c r="L26" s="30"/>
+      <c r="M26" s="27"/>
+      <c r="N26" s="27"/>
+      <c r="O26" s="27"/>
+      <c r="P26" s="27"/>
+      <c r="Q26" s="31"/>
+      <c r="R26" s="31"/>
+      <c r="S26" s="31"/>
+      <c r="T26" s="46"/>
+      <c r="U26" s="31"/>
+      <c r="V26" s="31"/>
+      <c r="W26" s="31"/>
+      <c r="X26" s="31"/>
+      <c r="Y26" s="31"/>
+      <c r="Z26" s="25"/>
+      <c r="AA26" s="25"/>
+      <c r="AB26" s="25"/>
     </row>
     <row r="27" spans="1:28" ht="48" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="93"/>
-      <c r="B27" s="93"/>
-      <c r="C27" s="93"/>
-      <c r="D27" s="93"/>
-      <c r="E27" s="93"/>
-      <c r="F27" s="93"/>
-      <c r="G27" s="93"/>
-      <c r="H27" s="30"/>
-      <c r="I27" s="29"/>
-      <c r="J27" s="30"/>
-      <c r="K27" s="31"/>
-      <c r="L27" s="32"/>
-      <c r="M27" s="29"/>
-      <c r="N27" s="29"/>
-      <c r="O27" s="29"/>
-      <c r="P27" s="29"/>
-      <c r="Q27" s="33"/>
-      <c r="R27" s="33"/>
-      <c r="S27" s="33"/>
-      <c r="T27" s="48"/>
-      <c r="U27" s="33"/>
-      <c r="V27" s="33"/>
-      <c r="W27" s="33"/>
-      <c r="X27" s="33"/>
-      <c r="Y27" s="33"/>
-      <c r="Z27" s="26"/>
-      <c r="AA27" s="26"/>
-      <c r="AB27" s="26"/>
+      <c r="A27" s="49"/>
+      <c r="B27" s="49"/>
+      <c r="C27" s="49"/>
+      <c r="D27" s="49"/>
+      <c r="E27" s="49"/>
+      <c r="F27" s="49"/>
+      <c r="G27" s="49"/>
+      <c r="H27" s="28"/>
+      <c r="I27" s="27"/>
+      <c r="J27" s="28"/>
+      <c r="K27" s="29"/>
+      <c r="L27" s="30"/>
+      <c r="M27" s="27"/>
+      <c r="N27" s="27"/>
+      <c r="O27" s="27"/>
+      <c r="P27" s="27"/>
+      <c r="Q27" s="31"/>
+      <c r="R27" s="31"/>
+      <c r="S27" s="31"/>
+      <c r="T27" s="46"/>
+      <c r="U27" s="31"/>
+      <c r="V27" s="31"/>
+      <c r="W27" s="31"/>
+      <c r="X27" s="31"/>
+      <c r="Y27" s="31"/>
+      <c r="Z27" s="25"/>
+      <c r="AA27" s="25"/>
+      <c r="AB27" s="25"/>
     </row>
     <row r="28" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="26"/>
-      <c r="B28" s="26"/>
-      <c r="C28" s="26"/>
-      <c r="D28" s="26"/>
-      <c r="E28" s="26"/>
-      <c r="F28" s="26"/>
-      <c r="G28" s="26"/>
-      <c r="H28" s="26"/>
-      <c r="I28" s="26"/>
-      <c r="J28" s="26"/>
-      <c r="K28" s="26"/>
-      <c r="L28" s="26"/>
-      <c r="M28" s="26"/>
-      <c r="N28" s="26"/>
-      <c r="O28" s="26"/>
-      <c r="P28" s="26"/>
-      <c r="Q28" s="26"/>
-      <c r="R28" s="26"/>
-      <c r="S28" s="26"/>
-      <c r="T28" s="26"/>
-      <c r="U28" s="26"/>
-      <c r="V28" s="26"/>
-      <c r="W28" s="26"/>
-      <c r="X28" s="26"/>
-      <c r="Y28" s="26"/>
-      <c r="Z28" s="26"/>
-      <c r="AA28" s="26"/>
-      <c r="AB28" s="26"/>
+      <c r="A28" s="25"/>
+      <c r="B28" s="25"/>
+      <c r="C28" s="25"/>
+      <c r="D28" s="25"/>
+      <c r="E28" s="25"/>
+      <c r="F28" s="25"/>
+      <c r="G28" s="25"/>
+      <c r="H28" s="25"/>
+      <c r="I28" s="25"/>
+      <c r="J28" s="25"/>
+      <c r="K28" s="25"/>
+      <c r="L28" s="25"/>
+      <c r="M28" s="25"/>
+      <c r="N28" s="25"/>
+      <c r="O28" s="25"/>
+      <c r="P28" s="25"/>
+      <c r="Q28" s="25"/>
+      <c r="R28" s="25"/>
+      <c r="S28" s="25"/>
+      <c r="T28" s="25"/>
+      <c r="U28" s="25"/>
+      <c r="V28" s="25"/>
+      <c r="W28" s="25"/>
+      <c r="X28" s="25"/>
+      <c r="Y28" s="25"/>
+      <c r="Z28" s="25"/>
+      <c r="AA28" s="25"/>
+      <c r="AB28" s="25"/>
     </row>
     <row r="29" spans="1:28" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="26"/>
-      <c r="B29" s="26"/>
-      <c r="C29" s="26"/>
-      <c r="D29" s="26"/>
-      <c r="E29" s="26"/>
-      <c r="F29" s="26"/>
-      <c r="G29" s="26"/>
-      <c r="H29" s="26"/>
-      <c r="I29" s="26"/>
-      <c r="J29" s="26"/>
-      <c r="K29" s="26"/>
-      <c r="L29" s="26"/>
-      <c r="M29" s="26"/>
-      <c r="N29" s="26"/>
-      <c r="O29" s="26"/>
-      <c r="P29" s="26"/>
-      <c r="Q29" s="26"/>
-      <c r="R29" s="26"/>
-      <c r="S29" s="26"/>
-      <c r="T29" s="26"/>
-      <c r="U29" s="26"/>
-      <c r="V29" s="26"/>
-      <c r="W29" s="26"/>
-      <c r="X29" s="26"/>
-      <c r="Y29" s="26"/>
-      <c r="Z29" s="26"/>
-      <c r="AA29" s="47"/>
-      <c r="AB29" s="26"/>
+      <c r="A29" s="25"/>
+      <c r="B29" s="25"/>
+      <c r="C29" s="25"/>
+      <c r="D29" s="25"/>
+      <c r="E29" s="25"/>
+      <c r="F29" s="25"/>
+      <c r="G29" s="25"/>
+      <c r="H29" s="25"/>
+      <c r="I29" s="25"/>
+      <c r="J29" s="25"/>
+      <c r="K29" s="25"/>
+      <c r="L29" s="25"/>
+      <c r="M29" s="25"/>
+      <c r="N29" s="25"/>
+      <c r="O29" s="25"/>
+      <c r="P29" s="25"/>
+      <c r="Q29" s="25"/>
+      <c r="R29" s="25"/>
+      <c r="S29" s="25"/>
+      <c r="T29" s="25"/>
+      <c r="U29" s="25"/>
+      <c r="V29" s="25"/>
+      <c r="W29" s="25"/>
+      <c r="X29" s="25"/>
+      <c r="Y29" s="25"/>
+      <c r="Z29" s="25"/>
+      <c r="AA29" s="45"/>
+      <c r="AB29" s="25"/>
     </row>
     <row r="30" spans="1:28" ht="26.25" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A30" s="34"/>
-      <c r="B30" s="26"/>
-      <c r="C30" s="26"/>
-      <c r="D30" s="26"/>
-      <c r="E30" s="26"/>
-      <c r="F30" s="26"/>
-      <c r="G30" s="26"/>
-      <c r="H30" s="26"/>
-      <c r="I30" s="26"/>
-      <c r="J30" s="26"/>
-      <c r="K30" s="35"/>
-      <c r="L30" s="35"/>
-      <c r="M30" s="35"/>
-      <c r="N30" s="35"/>
-      <c r="O30" s="49" t="s">
+      <c r="A30" s="32"/>
+      <c r="B30" s="25"/>
+      <c r="C30" s="25"/>
+      <c r="D30" s="25"/>
+      <c r="E30" s="25"/>
+      <c r="F30" s="25"/>
+      <c r="G30" s="25"/>
+      <c r="H30" s="25"/>
+      <c r="I30" s="25"/>
+      <c r="J30" s="25"/>
+      <c r="K30" s="33"/>
+      <c r="L30" s="33"/>
+      <c r="M30" s="33"/>
+      <c r="N30" s="33"/>
+      <c r="O30" s="47" t="s">
         <v>44</v>
       </c>
-      <c r="P30" s="50"/>
-      <c r="Q30" s="36"/>
-      <c r="R30" s="36"/>
-      <c r="S30" s="36"/>
-      <c r="T30" s="36"/>
-      <c r="U30" s="36"/>
-      <c r="V30" s="36"/>
-      <c r="W30" s="36"/>
-      <c r="X30" s="36"/>
-      <c r="Y30" s="36"/>
+      <c r="P30" s="48"/>
+      <c r="Q30" s="34"/>
+      <c r="R30" s="34"/>
+      <c r="S30" s="34"/>
+      <c r="T30" s="34"/>
+      <c r="U30" s="34"/>
+      <c r="V30" s="34"/>
+      <c r="W30" s="34"/>
+      <c r="X30" s="34"/>
+      <c r="Y30" s="99"/>
     </row>
     <row r="31" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A31" s="26"/>
-      <c r="B31" s="26"/>
-      <c r="C31" s="26"/>
-      <c r="D31" s="26"/>
-      <c r="E31" s="26"/>
-      <c r="F31" s="26"/>
-      <c r="G31" s="26"/>
-      <c r="H31" s="26"/>
-      <c r="I31" s="26"/>
-      <c r="J31" s="26"/>
-      <c r="K31" s="26"/>
-      <c r="L31" s="26"/>
-      <c r="M31" s="26"/>
-      <c r="N31" s="26"/>
-      <c r="O31" s="26"/>
-      <c r="P31" s="26"/>
-      <c r="Q31" s="26"/>
-      <c r="R31" s="26"/>
-      <c r="S31" s="26"/>
-      <c r="T31" s="26"/>
-      <c r="U31" s="26"/>
-      <c r="V31" s="26"/>
-      <c r="W31" s="26"/>
-      <c r="X31" s="26"/>
-      <c r="Y31" s="26"/>
+      <c r="A31" s="25"/>
+      <c r="B31" s="25"/>
+      <c r="C31" s="25"/>
+      <c r="D31" s="25"/>
+      <c r="E31" s="25"/>
+      <c r="F31" s="25"/>
+      <c r="G31" s="25"/>
+      <c r="H31" s="25"/>
+      <c r="I31" s="25"/>
+      <c r="J31" s="25"/>
+      <c r="K31" s="25"/>
+      <c r="L31" s="25"/>
+      <c r="M31" s="25"/>
+      <c r="N31" s="25"/>
+      <c r="O31" s="25"/>
+      <c r="P31" s="25"/>
+      <c r="Q31" s="25"/>
+      <c r="R31" s="25"/>
+      <c r="S31" s="25"/>
+      <c r="T31" s="25"/>
+      <c r="U31" s="25"/>
+      <c r="V31" s="25"/>
+      <c r="W31" s="25"/>
+      <c r="X31" s="25"/>
+      <c r="Y31" s="25"/>
     </row>
     <row r="32" spans="1:28" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A32" s="37" t="s">
+      <c r="A32" s="35" t="s">
         <v>45</v>
       </c>
-      <c r="B32" s="38"/>
-      <c r="C32" s="39"/>
-      <c r="D32" s="26"/>
-      <c r="E32" s="26"/>
-      <c r="F32" s="26"/>
-      <c r="G32" s="26"/>
-      <c r="H32" s="26"/>
-      <c r="I32" s="26"/>
-      <c r="J32" s="26"/>
-      <c r="K32" s="26"/>
-      <c r="L32" s="26"/>
-      <c r="M32" s="26"/>
-      <c r="N32" s="26"/>
-      <c r="O32" s="26"/>
-      <c r="P32" s="26"/>
-      <c r="Q32" s="26"/>
-      <c r="R32" s="26"/>
-      <c r="S32" s="40"/>
-      <c r="T32" s="41"/>
-      <c r="U32" s="41"/>
-      <c r="V32" s="41"/>
-      <c r="W32" s="41"/>
-      <c r="X32" s="41"/>
-      <c r="Y32" s="42"/>
+      <c r="B32" s="36"/>
+      <c r="C32" s="37"/>
+      <c r="D32" s="25"/>
+      <c r="E32" s="25"/>
+      <c r="F32" s="25"/>
+      <c r="G32" s="25"/>
+      <c r="H32" s="25"/>
+      <c r="I32" s="25"/>
+      <c r="J32" s="25"/>
+      <c r="K32" s="25"/>
+      <c r="L32" s="25"/>
+      <c r="M32" s="25"/>
+      <c r="N32" s="25"/>
+      <c r="O32" s="25"/>
+      <c r="P32" s="25"/>
+      <c r="Q32" s="25"/>
+      <c r="R32" s="25"/>
+      <c r="S32" s="38"/>
+      <c r="T32" s="39"/>
+      <c r="U32" s="39"/>
+      <c r="V32" s="39"/>
+      <c r="W32" s="39"/>
+      <c r="X32" s="39"/>
+      <c r="Y32" s="40"/>
     </row>
     <row r="33" spans="1:25" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A33" s="38"/>
-      <c r="B33" s="38"/>
-      <c r="C33" s="39"/>
-      <c r="D33" s="26"/>
-      <c r="E33" s="26"/>
-      <c r="F33" s="26"/>
-      <c r="G33" s="26"/>
-      <c r="H33" s="26"/>
-      <c r="I33" s="26"/>
-      <c r="J33" s="26"/>
-      <c r="K33" s="26"/>
-      <c r="L33" s="26"/>
-      <c r="M33" s="26"/>
-      <c r="N33" s="26"/>
-      <c r="O33" s="26"/>
-      <c r="P33" s="26"/>
-      <c r="Q33" s="34"/>
-      <c r="R33" s="34"/>
-      <c r="S33" s="40"/>
-      <c r="T33" s="41"/>
-      <c r="U33" s="41"/>
-      <c r="V33" s="41"/>
-      <c r="W33" s="41"/>
-      <c r="X33" s="41"/>
-      <c r="Y33" s="42"/>
+      <c r="A33" s="36"/>
+      <c r="B33" s="36"/>
+      <c r="C33" s="37"/>
+      <c r="D33" s="25"/>
+      <c r="E33" s="25"/>
+      <c r="F33" s="25"/>
+      <c r="G33" s="25"/>
+      <c r="H33" s="25"/>
+      <c r="I33" s="25"/>
+      <c r="J33" s="25"/>
+      <c r="K33" s="25"/>
+      <c r="L33" s="25"/>
+      <c r="M33" s="25"/>
+      <c r="N33" s="25"/>
+      <c r="O33" s="25"/>
+      <c r="P33" s="25"/>
+      <c r="Q33" s="32"/>
+      <c r="R33" s="32"/>
+      <c r="S33" s="38"/>
+      <c r="T33" s="39"/>
+      <c r="U33" s="39"/>
+      <c r="V33" s="39"/>
+      <c r="W33" s="39"/>
+      <c r="X33" s="39"/>
+      <c r="Y33" s="40"/>
     </row>
     <row r="34" spans="1:25" ht="20.25" x14ac:dyDescent="0.3">
-      <c r="A34" s="43" t="s">
+      <c r="A34" s="41" t="s">
         <v>46</v>
       </c>
-      <c r="B34" s="38"/>
-      <c r="C34" s="39"/>
-      <c r="D34" s="26"/>
-      <c r="E34" s="26"/>
-      <c r="F34" s="26"/>
-      <c r="G34" s="90" t="s">
+      <c r="B34" s="36"/>
+      <c r="C34" s="37"/>
+      <c r="D34" s="25"/>
+      <c r="E34" s="25"/>
+      <c r="F34" s="25"/>
+      <c r="G34" s="96" t="s">
         <v>47</v>
       </c>
-      <c r="H34" s="90"/>
-      <c r="I34" s="26"/>
-      <c r="J34" s="26"/>
-      <c r="K34" s="26"/>
-      <c r="L34" s="44"/>
-      <c r="M34" s="90" t="s">
+      <c r="H34" s="96"/>
+      <c r="I34" s="25"/>
+      <c r="J34" s="25"/>
+      <c r="K34" s="25"/>
+      <c r="L34" s="42"/>
+      <c r="M34" s="96" t="s">
         <v>48</v>
       </c>
-      <c r="N34" s="90"/>
-      <c r="O34" s="26"/>
-      <c r="P34" s="26"/>
-      <c r="Q34" s="26"/>
-      <c r="R34" s="26"/>
-      <c r="S34" s="40"/>
-      <c r="T34" s="41"/>
-      <c r="U34" s="41"/>
-      <c r="V34" s="41"/>
-      <c r="W34" s="41"/>
-      <c r="X34" s="41"/>
-      <c r="Y34" s="42"/>
+      <c r="N34" s="96"/>
+      <c r="O34" s="25"/>
+      <c r="P34" s="25"/>
+      <c r="Q34" s="25"/>
+      <c r="R34" s="25"/>
+      <c r="S34" s="38"/>
+      <c r="T34" s="39"/>
+      <c r="U34" s="39"/>
+      <c r="V34" s="39"/>
+      <c r="W34" s="39"/>
+      <c r="X34" s="39"/>
+      <c r="Y34" s="40"/>
     </row>
     <row r="35" spans="1:25" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="38"/>
-      <c r="B35" s="38"/>
-      <c r="C35" s="39"/>
-      <c r="D35" s="26"/>
-      <c r="O35" s="26"/>
-      <c r="P35" s="26"/>
-      <c r="S35" s="26"/>
-      <c r="T35" s="26"/>
-      <c r="U35" s="26"/>
-      <c r="V35" s="26"/>
-      <c r="W35" s="26"/>
-      <c r="X35" s="26"/>
-      <c r="Y35" s="26"/>
+      <c r="A35" s="36"/>
+      <c r="B35" s="36"/>
+      <c r="C35" s="37"/>
+      <c r="D35" s="25"/>
+      <c r="O35" s="25"/>
+      <c r="P35" s="25"/>
+      <c r="S35" s="25"/>
+      <c r="T35" s="25"/>
+      <c r="U35" s="25"/>
+      <c r="V35" s="25"/>
+      <c r="W35" s="25"/>
+      <c r="X35" s="25"/>
+      <c r="Y35" s="25"/>
     </row>
     <row r="36" spans="1:25" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="43" t="str">
+      <c r="A36" s="41" t="str">
         <f>+'[1]ANEXO NP1'!A78</f>
         <v>MES: FEBRERO   AÑO: 2025</v>
       </c>
-      <c r="B36" s="38"/>
-      <c r="C36" s="39"/>
-      <c r="D36" s="26"/>
-      <c r="E36" s="26"/>
-      <c r="F36" s="26"/>
-      <c r="G36" s="26"/>
-      <c r="H36" s="26"/>
-      <c r="I36" s="26"/>
-      <c r="J36" s="26"/>
-      <c r="K36" s="45"/>
-      <c r="L36" s="26"/>
-      <c r="M36" s="45"/>
+      <c r="B36" s="36"/>
+      <c r="C36" s="37"/>
+      <c r="D36" s="25"/>
+      <c r="E36" s="25"/>
+      <c r="F36" s="25"/>
+      <c r="G36" s="25"/>
+      <c r="H36" s="25"/>
+      <c r="I36" s="25"/>
+      <c r="J36" s="25"/>
+      <c r="K36" s="43"/>
+      <c r="L36" s="25"/>
+      <c r="M36" s="43"/>
       <c r="N36" s="1"/>
-      <c r="O36" s="45"/>
-      <c r="P36" s="26"/>
-      <c r="S36" s="26"/>
+      <c r="O36" s="43"/>
+      <c r="P36" s="25"/>
+      <c r="S36" s="25"/>
       <c r="T36" s="1"/>
       <c r="U36" s="1"/>
       <c r="V36" s="1"/>
       <c r="W36" s="1"/>
       <c r="X36" s="1"/>
-      <c r="Y36" s="26"/>
+      <c r="Y36" s="25"/>
     </row>
     <row r="37" spans="1:25" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="1"/>
-      <c r="B37" s="26"/>
-      <c r="K37" s="26"/>
-      <c r="L37" s="26"/>
-      <c r="M37" s="26"/>
-      <c r="N37" s="26"/>
-      <c r="O37" s="26"/>
-      <c r="P37" s="26"/>
-      <c r="S37" s="26"/>
-      <c r="T37" s="26"/>
-      <c r="U37" s="26"/>
-      <c r="V37" s="26"/>
-      <c r="W37" s="26"/>
-      <c r="X37" s="26"/>
-      <c r="Y37" s="26"/>
+      <c r="B37" s="25"/>
+      <c r="K37" s="25"/>
+      <c r="L37" s="25"/>
+      <c r="M37" s="25"/>
+      <c r="N37" s="25"/>
+      <c r="O37" s="25"/>
+      <c r="P37" s="25"/>
+      <c r="S37" s="25"/>
+      <c r="T37" s="25"/>
+      <c r="U37" s="25"/>
+      <c r="V37" s="25"/>
+      <c r="W37" s="25"/>
+      <c r="X37" s="25"/>
+      <c r="Y37" s="25"/>
     </row>
     <row r="38" spans="1:25" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="1"/>
-      <c r="B38" s="26"/>
-      <c r="C38" s="26"/>
-      <c r="D38" s="26"/>
-      <c r="E38" s="26"/>
-      <c r="F38" s="26"/>
-      <c r="G38" s="26"/>
-      <c r="H38" s="26"/>
-      <c r="I38" s="26"/>
-      <c r="J38" s="26"/>
-      <c r="K38" s="26"/>
-      <c r="L38" s="26"/>
-      <c r="M38" s="26"/>
-      <c r="N38" s="26"/>
-      <c r="O38" s="26"/>
-      <c r="P38" s="26"/>
-      <c r="Q38" s="26"/>
-      <c r="R38" s="26"/>
-      <c r="S38" s="26"/>
-      <c r="T38" s="26"/>
-      <c r="U38" s="26"/>
-      <c r="V38" s="26"/>
-      <c r="W38" s="26"/>
-      <c r="X38" s="26"/>
-      <c r="Y38" s="46" t="s">
+      <c r="B38" s="25"/>
+      <c r="C38" s="25"/>
+      <c r="D38" s="25"/>
+      <c r="E38" s="25"/>
+      <c r="F38" s="25"/>
+      <c r="G38" s="25"/>
+      <c r="H38" s="25"/>
+      <c r="I38" s="25"/>
+      <c r="J38" s="25"/>
+      <c r="K38" s="25"/>
+      <c r="L38" s="25"/>
+      <c r="M38" s="25"/>
+      <c r="N38" s="25"/>
+      <c r="O38" s="25"/>
+      <c r="P38" s="25"/>
+      <c r="Q38" s="25"/>
+      <c r="R38" s="25"/>
+      <c r="S38" s="25"/>
+      <c r="T38" s="25"/>
+      <c r="U38" s="25"/>
+      <c r="V38" s="25"/>
+      <c r="W38" s="25"/>
+      <c r="X38" s="25"/>
+      <c r="Y38" s="44" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="39" spans="1:25" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
-  <mergeCells count="32">
+  <mergeCells count="33">
     <mergeCell ref="G34:H34"/>
     <mergeCell ref="M34:N34"/>
     <mergeCell ref="T7:T10"/>
@@ -3381,6 +3251,7 @@
     <mergeCell ref="I9:I10"/>
     <mergeCell ref="K9:K10"/>
     <mergeCell ref="L9:O9"/>
+    <mergeCell ref="P7:P10"/>
     <mergeCell ref="A7:A10"/>
     <mergeCell ref="B7:B10"/>
     <mergeCell ref="C7:C10"/>

</xml_diff>